<commit_message>
chore: prepare main for local IDC cron test
Remove the current-release generated outputs from the local main baseline while keeping the files needed for the scheduled IDC automation available locally.
</commit_message>
<xml_diff>
--- a/data/processed/idc_data.xlsx
+++ b/data/processed/idc_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:E181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -847,13 +847,13 @@
         <v>0.2272727272727273</v>
       </c>
       <c r="C37" t="n">
-        <v>0.05882352941176449</v>
+        <v>0.0588235294117644</v>
       </c>
       <c r="D37" t="n">
         <v>0.8309695443551434</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3723552670132118</v>
+        <v>0.3723552670132117</v>
       </c>
     </row>
     <row r="38">
@@ -866,7 +866,7 @@
         <v>0.1818181818181812</v>
       </c>
       <c r="C38" t="n">
-        <v>0.05882352941176449</v>
+        <v>0.0588235294117644</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
@@ -885,7 +885,7 @@
         <v>0.1818181818181812</v>
       </c>
       <c r="C39" t="n">
-        <v>0.05882352941176449</v>
+        <v>0.0588235294117644</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
         <v>0.2727272727272735</v>
       </c>
       <c r="C41" t="n">
-        <v>0.05882352941176449</v>
+        <v>0.0588235294117644</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.318181818181818</v>
+        <v>0.3181818181818179</v>
       </c>
       <c r="C42" t="n">
         <v>0.1176470588235295</v>
@@ -948,7 +948,7 @@
         <v>0.8324983307105308</v>
       </c>
       <c r="E42" t="n">
-        <v>0.4227757359052928</v>
+        <v>0.4227757359052927</v>
       </c>
     </row>
     <row r="43">
@@ -999,7 +999,7 @@
         <v>0.2727272727272735</v>
       </c>
       <c r="C45" t="n">
-        <v>0.05882352941176449</v>
+        <v>0.0588235294117644</v>
       </c>
       <c r="D45" t="n">
         <v>0.7830522467498834</v>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.4090909090909086</v>
+        <v>0.4090909090909085</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -1059,10 +1059,10 @@
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4546540657780138</v>
+        <v>0.4546540657780137</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4242786279866109</v>
+        <v>0.4242786279866108</v>
       </c>
     </row>
     <row r="49">
@@ -1110,13 +1110,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.9545454545454555</v>
+        <v>0.9545454545454556</v>
       </c>
       <c r="C51" t="n">
-        <v>0.04999999999999982</v>
+        <v>0.0499999999999998</v>
       </c>
       <c r="D51" t="n">
-        <v>0.9191340608899673</v>
+        <v>0.9191340608899672</v>
       </c>
       <c r="E51" t="n">
         <v>0.6412265051451409</v>
@@ -1129,10 +1129,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.9545454545454555</v>
+        <v>0.9545454545454556</v>
       </c>
       <c r="C52" t="n">
-        <v>0.1000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D52" t="n">
         <v>0.9354739862101402</v>
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.9545454545454555</v>
+        <v>0.9545454545454556</v>
       </c>
       <c r="C53" t="n">
-        <v>0.04999999999999982</v>
+        <v>0.0499999999999998</v>
       </c>
       <c r="D53" t="n">
-        <v>0.9759592328097707</v>
+        <v>0.9759592328097708</v>
       </c>
       <c r="E53" t="n">
         <v>0.6601682291184087</v>
@@ -1170,7 +1170,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>0.1000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D54" t="n">
         <v>0.8883007681125101</v>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.4400000000000006</v>
+        <v>0.4400000000000005</v>
       </c>
       <c r="C60" t="n">
         <v>0.5</v>
@@ -1325,7 +1325,7 @@
         <v>0.5</v>
       </c>
       <c r="D62" t="n">
-        <v>0.9725506805246665</v>
+        <v>0.9725506805246664</v>
       </c>
       <c r="E62" t="n">
         <v>0.6908502268415555</v>
@@ -1363,7 +1363,7 @@
         <v>0.5499999999999998</v>
       </c>
       <c r="D64" t="n">
-        <v>0.9749943209794701</v>
+        <v>0.97499432097947</v>
       </c>
       <c r="E64" t="n">
         <v>0.7349981069931566</v>
@@ -1382,7 +1382,7 @@
         <v>0.5</v>
       </c>
       <c r="D65" t="n">
-        <v>0.9310890047696613</v>
+        <v>0.9310890047696612</v>
       </c>
       <c r="E65" t="n">
         <v>0.7170296682565538</v>
@@ -1499,7 +1499,7 @@
         <v>0.1978798745881518</v>
       </c>
       <c r="E71" t="n">
-        <v>0.3326266248627173</v>
+        <v>0.3326266248627172</v>
       </c>
     </row>
     <row r="72">
@@ -1556,7 +1556,7 @@
         <v>0.3628231483643701</v>
       </c>
       <c r="E74" t="n">
-        <v>0.33094104945479</v>
+        <v>0.3309410494547899</v>
       </c>
     </row>
     <row r="75">
@@ -1566,13 +1566,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.1200000000000003</v>
+        <v>0.1200000000000002</v>
       </c>
       <c r="C75" t="n">
         <v>0.2999999999999998</v>
       </c>
       <c r="D75" t="n">
-        <v>0.4356421767454646</v>
+        <v>0.4356421767454645</v>
       </c>
       <c r="E75" t="n">
         <v>0.2852140589151549</v>
@@ -1629,10 +1629,10 @@
         <v>0.25</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2399283557599176</v>
+        <v>0.2399283557599175</v>
       </c>
       <c r="E78" t="n">
-        <v>0.2003464889570097</v>
+        <v>0.2003464889570096</v>
       </c>
     </row>
     <row r="79">
@@ -1648,7 +1648,7 @@
         <v>0.25</v>
       </c>
       <c r="D79" t="n">
-        <v>0.1629527256875273</v>
+        <v>0.1629527256875272</v>
       </c>
       <c r="E79" t="n">
         <v>0.2117249826365829</v>
@@ -1670,7 +1670,7 @@
         <v>0.1102481552651509</v>
       </c>
       <c r="E80" t="n">
-        <v>0.2021814838538158</v>
+        <v>0.2021814838538157</v>
       </c>
     </row>
     <row r="81">
@@ -1702,7 +1702,7 @@
         <v>0.1111111111111114</v>
       </c>
       <c r="C82" t="n">
-        <v>0.1000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.03703703703703626</v>
+        <v>0.0370370370370362</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
@@ -1727,7 +1727,7 @@
         <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>0.01234567901234542</v>
+        <v>0.0123456790123454</v>
       </c>
     </row>
     <row r="84">
@@ -1743,10 +1743,10 @@
         <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>0.07217268456268752</v>
+        <v>0.07217268456268749</v>
       </c>
       <c r="E84" t="n">
-        <v>0.02405756152089584</v>
+        <v>0.0240575615208958</v>
       </c>
     </row>
     <row r="85">
@@ -1765,7 +1765,7 @@
         <v>0.2373397296057668</v>
       </c>
       <c r="E85" t="n">
-        <v>0.07911324320192227</v>
+        <v>0.0791132432019222</v>
       </c>
     </row>
     <row r="86">
@@ -1775,16 +1775,16 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.03571428571428621</v>
+        <v>0.0357142857142862</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
       </c>
       <c r="D86" t="n">
-        <v>0.1736702105847082</v>
+        <v>0.1736702105847081</v>
       </c>
       <c r="E86" t="n">
-        <v>0.06979483209966479</v>
+        <v>0.06979483209966469</v>
       </c>
     </row>
     <row r="87">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.1428571428571436</v>
+        <v>0.1428571428571435</v>
       </c>
       <c r="C87" t="n">
         <v>0</v>
@@ -1819,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="D88" t="n">
-        <v>0.1512087838932729</v>
+        <v>0.1512087838932728</v>
       </c>
       <c r="E88" t="n">
         <v>0.1337362612977575</v>
@@ -1838,10 +1838,10 @@
         <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>0.175105132324621</v>
+        <v>0.1751051323246209</v>
       </c>
       <c r="E89" t="n">
-        <v>0.1655112345843977</v>
+        <v>0.1655112345843976</v>
       </c>
     </row>
     <row r="90">
@@ -1854,13 +1854,13 @@
         <v>0.2142857142857147</v>
       </c>
       <c r="C90" t="n">
-        <v>0.04347826086956506</v>
+        <v>0.043478260869565</v>
       </c>
       <c r="D90" t="n">
-        <v>0.09045990357805485</v>
+        <v>0.09045990357805481</v>
       </c>
       <c r="E90" t="n">
-        <v>0.1160746262444449</v>
+        <v>0.1160746262444448</v>
       </c>
     </row>
     <row r="91">
@@ -1870,16 +1870,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.1071428571428574</v>
+        <v>0.1071428571428573</v>
       </c>
       <c r="C91" t="n">
-        <v>0.04347826086956506</v>
+        <v>0.043478260869565</v>
       </c>
       <c r="D91" t="n">
-        <v>0.03831298161070876</v>
+        <v>0.0383129816107087</v>
       </c>
       <c r="E91" t="n">
-        <v>0.06297803320771041</v>
+        <v>0.06297803320771039</v>
       </c>
     </row>
     <row r="92">
@@ -1889,16 +1889,16 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.1428571428571436</v>
+        <v>0.1428571428571435</v>
       </c>
       <c r="C92" t="n">
         <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>0.01791067967242742</v>
+        <v>0.0179106796724274</v>
       </c>
       <c r="E92" t="n">
-        <v>0.05358927417652367</v>
+        <v>0.0535892741765236</v>
       </c>
     </row>
     <row r="93">
@@ -1908,16 +1908,16 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.1071428571428574</v>
+        <v>0.1071428571428573</v>
       </c>
       <c r="C93" t="n">
         <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>0.04898742351801629</v>
+        <v>0.0489874235180162</v>
       </c>
       <c r="E93" t="n">
-        <v>0.05204342688695789</v>
+        <v>0.0520434268869578</v>
       </c>
     </row>
     <row r="94">
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="D94" t="n">
-        <v>0.006163490244665353</v>
+        <v>0.0061634902446653</v>
       </c>
       <c r="E94" t="n">
-        <v>0.06157830627203129</v>
+        <v>0.0615783062720312</v>
       </c>
     </row>
     <row r="95">
@@ -1971,10 +1971,10 @@
         <v>0</v>
       </c>
       <c r="D96" t="n">
-        <v>0.1239804710481171</v>
+        <v>0.123980471048117</v>
       </c>
       <c r="E96" t="n">
-        <v>0.1484696808255631</v>
+        <v>0.148469680825563</v>
       </c>
     </row>
     <row r="97">
@@ -1990,7 +1990,7 @@
         <v>0</v>
       </c>
       <c r="D97" t="n">
-        <v>0.2448778821631855</v>
+        <v>0.2448778821631854</v>
       </c>
       <c r="E97" t="n">
         <v>0.2125783416734429</v>
@@ -2012,7 +2012,7 @@
         <v>0.2320166827458945</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2082912752010126</v>
+        <v>0.2082912752010125</v>
       </c>
     </row>
     <row r="99">
@@ -2028,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="D99" t="n">
-        <v>0.2854673416493079</v>
+        <v>0.2854673416493078</v>
       </c>
       <c r="E99" t="n">
         <v>0.2856319710259599</v>
@@ -2044,13 +2044,13 @@
         <v>0.6785714285714292</v>
       </c>
       <c r="C100" t="n">
-        <v>0.03999999999999986</v>
+        <v>0.0399999999999998</v>
       </c>
       <c r="D100" t="n">
         <v>0.2905293572727042</v>
       </c>
       <c r="E100" t="n">
-        <v>0.3363669286147111</v>
+        <v>0.336366928614711</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="C101" t="n">
-        <v>0.03999999999999986</v>
+        <v>0.0399999999999998</v>
       </c>
       <c r="D101" t="n">
         <v>0.3513175817075109</v>
@@ -2082,7 +2082,7 @@
         <v>0.8999999999999998</v>
       </c>
       <c r="C102" t="n">
-        <v>0.03999999999999986</v>
+        <v>0.0399999999999998</v>
       </c>
       <c r="D102" t="n">
         <v>0.2860368403049701</v>
@@ -2101,7 +2101,7 @@
         <v>0.9333333333333336</v>
       </c>
       <c r="C103" t="n">
-        <v>0.08000000000000007</v>
+        <v>0.08</v>
       </c>
       <c r="D103" t="n">
         <v>0.2805459391879865</v>
@@ -2123,7 +2123,7 @@
         <v>0.1199999999999999</v>
       </c>
       <c r="D104" t="n">
-        <v>0.2809435606936265</v>
+        <v>0.2809435606936264</v>
       </c>
       <c r="E104" t="n">
         <v>0.3558700757867643</v>
@@ -2164,7 +2164,7 @@
         <v>0.1981927225528276</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2393975741842758</v>
+        <v>0.2393975741842757</v>
       </c>
     </row>
     <row r="107">
@@ -2180,10 +2180,10 @@
         <v>0.1199999999999999</v>
       </c>
       <c r="D107" t="n">
-        <v>0.02479784971327119</v>
+        <v>0.0247978497132711</v>
       </c>
       <c r="E107" t="n">
-        <v>0.1371548387933127</v>
+        <v>0.1371548387933126</v>
       </c>
     </row>
     <row r="108">
@@ -2196,7 +2196,7 @@
         <v>0.2666666666666669</v>
       </c>
       <c r="C108" t="n">
-        <v>0.08000000000000007</v>
+        <v>0.08</v>
       </c>
       <c r="D108" t="n">
         <v>0.1035980211576326</v>
@@ -2215,10 +2215,10 @@
         <v>0.2333333333333331</v>
       </c>
       <c r="C109" t="n">
-        <v>0.1599999999999998</v>
+        <v>0.1599999999999997</v>
       </c>
       <c r="D109" t="n">
-        <v>0.2048299465559415</v>
+        <v>0.2048299465559414</v>
       </c>
       <c r="E109" t="n">
         <v>0.1993877599630914</v>
@@ -2253,13 +2253,13 @@
         <v>0.3999999999999997</v>
       </c>
       <c r="C111" t="n">
-        <v>0.32</v>
+        <v>0.3199999999999999</v>
       </c>
       <c r="D111" t="n">
         <v>0.4283229775251577</v>
       </c>
       <c r="E111" t="n">
-        <v>0.3827743258417192</v>
+        <v>0.3827743258417191</v>
       </c>
     </row>
     <row r="112">
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>0.3599999999999998</v>
+        <v>0.3599999999999997</v>
       </c>
       <c r="D112" t="n">
-        <v>0.3165758112709071</v>
+        <v>0.316575811270907</v>
       </c>
       <c r="E112" t="n">
         <v>0.2255252704236356</v>
@@ -2291,13 +2291,13 @@
         <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0.2399999999999999</v>
+        <v>0.2399999999999998</v>
       </c>
       <c r="D113" t="n">
         <v>0.1678060787477241</v>
       </c>
       <c r="E113" t="n">
-        <v>0.1359353595825747</v>
+        <v>0.1359353595825746</v>
       </c>
     </row>
     <row r="114">
@@ -2310,13 +2310,13 @@
         <v>0</v>
       </c>
       <c r="C114" t="n">
-        <v>0.1599999999999998</v>
+        <v>0.1599999999999997</v>
       </c>
       <c r="D114" t="n">
-        <v>0.01685373950402727</v>
+        <v>0.0168537395040272</v>
       </c>
       <c r="E114" t="n">
-        <v>0.05895124650134235</v>
+        <v>0.0589512465013423</v>
       </c>
     </row>
     <row r="115">
@@ -2329,13 +2329,13 @@
         <v>0</v>
       </c>
       <c r="C115" t="n">
-        <v>0.08000000000000007</v>
+        <v>0.08</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
       </c>
       <c r="E115" t="n">
-        <v>0.02666666666666669</v>
+        <v>0.0266666666666666</v>
       </c>
     </row>
     <row r="116">
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.05882352941176417</v>
+        <v>0.0588235294117641</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="E116" t="n">
-        <v>0.01960784313725472</v>
+        <v>0.0196078431372547</v>
       </c>
     </row>
     <row r="117">
@@ -2373,7 +2373,7 @@
         <v>0</v>
       </c>
       <c r="E117" t="n">
-        <v>0.05882352941176464</v>
+        <v>0.0588235294117646</v>
       </c>
     </row>
     <row r="118">
@@ -2411,7 +2411,7 @@
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>0.1568627450980392</v>
+        <v>0.1568627450980391</v>
       </c>
     </row>
     <row r="120">
@@ -2468,7 +2468,7 @@
         <v>0.2153533575103212</v>
       </c>
       <c r="E122" t="n">
-        <v>0.2482550407387346</v>
+        <v>0.2482550407387345</v>
       </c>
     </row>
     <row r="123">
@@ -2500,7 +2500,7 @@
         <v>0.6078431372549018</v>
       </c>
       <c r="C124" t="n">
-        <v>0.03124999999999989</v>
+        <v>0.0312499999999998</v>
       </c>
       <c r="D124" t="n">
         <v>0.2545599775084994</v>
@@ -2525,7 +2525,7 @@
         <v>0.2814720600383868</v>
       </c>
       <c r="E125" t="n">
-        <v>0.3029743468101813</v>
+        <v>0.3029743468101812</v>
       </c>
     </row>
     <row r="126">
@@ -2538,7 +2538,7 @@
         <v>0.7058823529411763</v>
       </c>
       <c r="C126" t="n">
-        <v>0.03124999999999989</v>
+        <v>0.0312499999999998</v>
       </c>
       <c r="D126" t="n">
         <v>0.2878714351788128</v>
@@ -2557,7 +2557,7 @@
         <v>0.7843137254901964</v>
       </c>
       <c r="C127" t="n">
-        <v>0.03124999999999989</v>
+        <v>0.0312499999999998</v>
       </c>
       <c r="D127" t="n">
         <v>0.3567797887508668</v>
@@ -2573,16 +2573,16 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.9607843137254903</v>
+        <v>0.9607843137254904</v>
       </c>
       <c r="C128" t="n">
-        <v>0.06250000000000006</v>
+        <v>0.0625</v>
       </c>
       <c r="D128" t="n">
         <v>0.4338893293994195</v>
       </c>
       <c r="E128" t="n">
-        <v>0.4857245477083033</v>
+        <v>0.4857245477083032</v>
       </c>
     </row>
     <row r="129">
@@ -2595,7 +2595,7 @@
         <v>1</v>
       </c>
       <c r="C129" t="n">
-        <v>0.06250000000000006</v>
+        <v>0.0625</v>
       </c>
       <c r="D129" t="n">
         <v>0.5109885971651589</v>
@@ -2614,7 +2614,7 @@
         <v>1</v>
       </c>
       <c r="C130" t="n">
-        <v>0.09374999999999994</v>
+        <v>0.0937499999999999</v>
       </c>
       <c r="D130" t="n">
         <v>0.5224447035496396</v>
@@ -2671,7 +2671,7 @@
         <v>0.9242424242424242</v>
       </c>
       <c r="C133" t="n">
-        <v>0.2187500000000001</v>
+        <v>0.21875</v>
       </c>
       <c r="D133" t="n">
         <v>0.7999634422509253</v>
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.9545454545454545</v>
+        <v>0.9545454545454544</v>
       </c>
       <c r="C137" t="n">
-        <v>0.3750000000000001</v>
+        <v>0.375</v>
       </c>
       <c r="D137" t="n">
         <v>0.8621984129111688</v>
@@ -2826,7 +2826,7 @@
         <v>0.5624999999999999</v>
       </c>
       <c r="D141" t="n">
-        <v>0.9434585701441283</v>
+        <v>0.9434585701441284</v>
       </c>
       <c r="E141" t="n">
         <v>0.8353195233813761</v>
@@ -2845,7 +2845,7 @@
         <v>0.5624999999999999</v>
       </c>
       <c r="D142" t="n">
-        <v>0.9341003903548799</v>
+        <v>0.93410039035488</v>
       </c>
       <c r="E142" t="n">
         <v>0.8322001301182933</v>
@@ -2883,7 +2883,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D144" t="n">
-        <v>0.9359548364085427</v>
+        <v>0.9359548364085428</v>
       </c>
       <c r="E144" t="n">
         <v>0.8640682788028475</v>
@@ -2921,7 +2921,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D146" t="n">
-        <v>0.9534504164253911</v>
+        <v>0.9534504164253912</v>
       </c>
       <c r="E146" t="n">
         <v>0.8699001388084637</v>
@@ -2962,7 +2962,7 @@
         <v>0.987505664722233</v>
       </c>
       <c r="E148" t="n">
-        <v>0.9020852215740777</v>
+        <v>0.9020852215740776</v>
       </c>
     </row>
     <row r="149">
@@ -3016,7 +3016,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D151" t="n">
-        <v>0.9045886593715887</v>
+        <v>0.9045886593715888</v>
       </c>
       <c r="E151" t="n">
         <v>0.8094361796298871</v>
@@ -3168,7 +3168,7 @@
         <v>0.46875</v>
       </c>
       <c r="D159" t="n">
-        <v>0.9710731241272009</v>
+        <v>0.9710731241272008</v>
       </c>
       <c r="E159" t="n">
         <v>0.7369691538255329</v>
@@ -3187,7 +3187,7 @@
         <v>0.46875</v>
       </c>
       <c r="D160" t="n">
-        <v>0.9526198528080617</v>
+        <v>0.9526198528080616</v>
       </c>
       <c r="E160" t="n">
         <v>0.7308180633858198</v>
@@ -3206,7 +3206,7 @@
         <v>0.4375000000000001</v>
       </c>
       <c r="D161" t="n">
-        <v>0.9347747781531663</v>
+        <v>0.9347747781531665</v>
       </c>
       <c r="E161" t="n">
         <v>0.7265012312719391</v>
@@ -3225,7 +3225,7 @@
         <v>0.46875</v>
       </c>
       <c r="D162" t="n">
-        <v>0.9185303003362743</v>
+        <v>0.9185303003362744</v>
       </c>
       <c r="E162" t="n">
         <v>0.7395352005136978</v>
@@ -3244,7 +3244,7 @@
         <v>0.46875</v>
       </c>
       <c r="D163" t="n">
-        <v>0.9405333228759577</v>
+        <v>0.9405333228759576</v>
       </c>
       <c r="E163" t="n">
         <v>0.7589177341313434</v>
@@ -3263,7 +3263,7 @@
         <v>0.4999999999999999</v>
       </c>
       <c r="D164" t="n">
-        <v>0.9823322045432281</v>
+        <v>0.982332204543228</v>
       </c>
       <c r="E164" t="n">
         <v>0.7792512970967387</v>
@@ -3282,7 +3282,7 @@
         <v>0.4375000000000001</v>
       </c>
       <c r="D165" t="n">
-        <v>0.9844349745515915</v>
+        <v>0.9844349745515916</v>
       </c>
       <c r="E165" t="n">
         <v>0.7591188870995266</v>
@@ -3317,7 +3317,7 @@
         <v>0.8915662650602411</v>
       </c>
       <c r="C167" t="n">
-        <v>0.3750000000000001</v>
+        <v>0.375</v>
       </c>
       <c r="D167" t="n">
         <v>0.908477471644922</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.9156626506024097</v>
+        <v>0.9156626506024096</v>
       </c>
       <c r="C168" t="n">
         <v>0.4999999999999999</v>
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.9397590361445783</v>
+        <v>0.9397590361445785</v>
       </c>
       <c r="C171" t="n">
         <v>0.625</v>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.9638554216867473</v>
+        <v>0.9638554216867472</v>
       </c>
       <c r="C172" t="n">
         <v>0.6875</v>
@@ -3453,7 +3453,7 @@
         <v>0.78125</v>
       </c>
       <c r="D174" t="n">
-        <v>0.9940035084602725</v>
+        <v>0.9940035084602724</v>
       </c>
       <c r="E174" t="n">
         <v>0.9090202457919784</v>
@@ -3529,10 +3529,10 @@
         <v>0.84375</v>
       </c>
       <c r="D178" t="n">
-        <v>0.9929551033202063</v>
+        <v>0.9929551033202064</v>
       </c>
       <c r="E178" t="n">
-        <v>0.9346988025560109</v>
+        <v>0.9346988025560108</v>
       </c>
     </row>
     <row r="179">
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.9891304347826085</v>
+        <v>0.9891304347826084</v>
       </c>
       <c r="C179" t="n">
         <v>0.8749999999999999</v>
@@ -3564,13 +3564,13 @@
         <v>1</v>
       </c>
       <c r="C180" t="n">
-        <v>0.9062500000000001</v>
+        <v>0.90625</v>
       </c>
       <c r="D180" t="n">
-        <v>0.9922248499806769</v>
+        <v>0.99175252624052</v>
       </c>
       <c r="E180" t="n">
-        <v>0.9661582833268924</v>
+        <v>0.9660008420801732</v>
       </c>
     </row>
     <row r="181">
@@ -3590,25 +3590,6 @@
       </c>
       <c r="E181" t="n">
         <v>1</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="B182" t="n">
-        <v>0.9684210526315788</v>
-      </c>
-      <c r="C182" t="n">
-        <v>0.9375</v>
-      </c>
-      <c r="D182" t="n">
-        <v>0.954831548220203</v>
-      </c>
-      <c r="E182" t="n">
-        <v>0.9535842002839273</v>
       </c>
     </row>
   </sheetData>
@@ -3622,7 +3603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D182"/>
+  <dimension ref="A1:D181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3660,7 +3641,7 @@
         <v>5.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2144837064952339</v>
+        <v>0.2144837064952338</v>
       </c>
     </row>
     <row r="3">
@@ -3676,7 +3657,7 @@
         <v>5.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.216318931938421</v>
+        <v>0.2163189319384209</v>
       </c>
     </row>
     <row r="4">
@@ -3708,7 +3689,7 @@
         <v>5.9</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2158826655184728</v>
+        <v>0.2158826655184727</v>
       </c>
     </row>
     <row r="6">
@@ -3772,7 +3753,7 @@
         <v>6.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2179910005812397</v>
+        <v>0.2179910005812396</v>
       </c>
     </row>
     <row r="10">
@@ -3788,7 +3769,7 @@
         <v>6.6</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2182622171978539</v>
+        <v>0.2182622171978538</v>
       </c>
     </row>
     <row r="11">
@@ -3804,7 +3785,7 @@
         <v>6.7</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2133141087974606</v>
+        <v>0.2133141087974605</v>
       </c>
     </row>
     <row r="12">
@@ -3868,7 +3849,7 @@
         <v>7.1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2221233325942454</v>
+        <v>0.2221233325942453</v>
       </c>
     </row>
     <row r="16">
@@ -3884,7 +3865,7 @@
         <v>7.2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.220769753883536</v>
+        <v>0.2207697538835359</v>
       </c>
     </row>
     <row r="17">
@@ -3900,7 +3881,7 @@
         <v>7.1</v>
       </c>
       <c r="D17" t="n">
-        <v>0.2197200510871163</v>
+        <v>0.2197200510871162</v>
       </c>
     </row>
     <row r="18">
@@ -3916,7 +3897,7 @@
         <v>7.2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.2177195914744852</v>
+        <v>0.2177195914744851</v>
       </c>
     </row>
     <row r="19">
@@ -4044,7 +4025,7 @@
         <v>6.6</v>
       </c>
       <c r="D26" t="n">
-        <v>0.2181028585196967</v>
+        <v>0.2181028585196966</v>
       </c>
     </row>
     <row r="27">
@@ -4076,7 +4057,7 @@
         <v>6.6</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2172222433013914</v>
+        <v>0.2172222433013913</v>
       </c>
     </row>
     <row r="29">
@@ -4092,7 +4073,7 @@
         <v>6.3</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2178010163122744</v>
+        <v>0.2178010163122743</v>
       </c>
     </row>
     <row r="30">
@@ -4124,7 +4105,7 @@
         <v>6.1</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2167167319171494</v>
+        <v>0.2167167319171493</v>
       </c>
     </row>
     <row r="32">
@@ -4172,7 +4153,7 @@
         <v>5.7</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2187602876319878</v>
+        <v>0.2187602876319877</v>
       </c>
     </row>
     <row r="35">
@@ -4220,7 +4201,7 @@
         <v>5.6</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2202994011171443</v>
+        <v>0.2202994011171442</v>
       </c>
     </row>
     <row r="38">
@@ -4236,7 +4217,7 @@
         <v>5.6</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2224782495762383</v>
+        <v>0.2224782495762382</v>
       </c>
     </row>
     <row r="39">
@@ -4252,7 +4233,7 @@
         <v>5.6</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2254332403816362</v>
+        <v>0.2254332403816361</v>
       </c>
     </row>
     <row r="40">
@@ -4268,7 +4249,7 @@
         <v>5.7</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2249205544331556</v>
+        <v>0.2249205544331555</v>
       </c>
     </row>
     <row r="41">
@@ -4284,7 +4265,7 @@
         <v>5.6</v>
       </c>
       <c r="D41" t="n">
-        <v>0.2274453362709764</v>
+        <v>0.2274453362709763</v>
       </c>
     </row>
     <row r="42">
@@ -4300,7 +4281,7 @@
         <v>5.7</v>
       </c>
       <c r="D42" t="n">
-        <v>0.2247464567387061</v>
+        <v>0.224746456738706</v>
       </c>
     </row>
     <row r="43">
@@ -4316,7 +4297,7 @@
         <v>5.7</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2248368217595582</v>
+        <v>0.2248368217595581</v>
       </c>
     </row>
     <row r="44">
@@ -4332,7 +4313,7 @@
         <v>5.7</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2254800353761997</v>
+        <v>0.2254800353761996</v>
       </c>
     </row>
     <row r="45">
@@ -4396,7 +4377,7 @@
         <v>5.3</v>
       </c>
       <c r="D48" t="n">
-        <v>0.2186584209756129</v>
+        <v>0.2186584209756128</v>
       </c>
     </row>
     <row r="49">
@@ -4460,7 +4441,7 @@
         <v>5.4</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2264056574507284</v>
+        <v>0.2264056574507283</v>
       </c>
     </row>
     <row r="53">
@@ -4556,7 +4537,7 @@
         <v>6</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2285970857885173</v>
+        <v>0.2285970857885172</v>
       </c>
     </row>
     <row r="59">
@@ -4732,7 +4713,7 @@
         <v>6.2</v>
       </c>
       <c r="D69" t="n">
-        <v>0.227739378996592</v>
+        <v>0.2277393789965919</v>
       </c>
     </row>
     <row r="70">
@@ -4812,7 +4793,7 @@
         <v>5.9</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2186286523599865</v>
+        <v>0.2186286523599864</v>
       </c>
     </row>
     <row r="75">
@@ -4844,7 +4825,7 @@
         <v>5.9</v>
       </c>
       <c r="D76" t="n">
-        <v>0.2191753307115642</v>
+        <v>0.2191753307115641</v>
       </c>
     </row>
     <row r="77">
@@ -4860,7 +4841,7 @@
         <v>5.7</v>
       </c>
       <c r="D77" t="n">
-        <v>0.2175911308009368</v>
+        <v>0.2175911308009367</v>
       </c>
     </row>
     <row r="78">
@@ -4876,7 +4857,7 @@
         <v>5.7</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2161574089217935</v>
+        <v>0.2161574089217934</v>
       </c>
     </row>
     <row r="79">
@@ -4892,7 +4873,7 @@
         <v>5.7</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2146095360080125</v>
+        <v>0.2146095360080124</v>
       </c>
     </row>
     <row r="80">
@@ -4908,7 +4889,7 @@
         <v>5.6</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2135497203635996</v>
+        <v>0.2135497203635995</v>
       </c>
     </row>
     <row r="81">
@@ -4956,7 +4937,7 @@
         <v>5.2</v>
       </c>
       <c r="D83" t="n">
-        <v>0.2027358661530098</v>
+        <v>0.2027358661530097</v>
       </c>
     </row>
     <row r="84">
@@ -4972,7 +4953,7 @@
         <v>5.2</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2048076210931714</v>
+        <v>0.2048076210931713</v>
       </c>
     </row>
     <row r="85">
@@ -5020,7 +5001,7 @@
         <v>5.1</v>
       </c>
       <c r="D87" t="n">
-        <v>0.2087065635519888</v>
+        <v>0.2087065635519887</v>
       </c>
     </row>
     <row r="88">
@@ -5036,7 +5017,7 @@
         <v>5</v>
       </c>
       <c r="D88" t="n">
-        <v>0.2070763939707692</v>
+        <v>0.2070763939707691</v>
       </c>
     </row>
     <row r="89">
@@ -5100,7 +5081,7 @@
         <v>4.9</v>
       </c>
       <c r="D92" t="n">
-        <v>0.2032500016506408</v>
+        <v>0.2032500016506407</v>
       </c>
     </row>
     <row r="93">
@@ -5116,7 +5097,7 @@
         <v>4.9</v>
       </c>
       <c r="D93" t="n">
-        <v>0.2041420759579269</v>
+        <v>0.2041420759579268</v>
       </c>
     </row>
     <row r="94">
@@ -5132,7 +5113,7 @@
         <v>4.8</v>
       </c>
       <c r="D94" t="n">
-        <v>0.2029127923881969</v>
+        <v>0.2029127923881968</v>
       </c>
     </row>
     <row r="95">
@@ -5196,7 +5177,7 @@
         <v>4.7</v>
       </c>
       <c r="D98" t="n">
-        <v>0.2058670578992161</v>
+        <v>0.205867057899216</v>
       </c>
     </row>
     <row r="99">
@@ -5260,7 +5241,7 @@
         <v>4.8</v>
       </c>
       <c r="D102" t="n">
-        <v>0.2076659636631001</v>
+        <v>0.2076659636631</v>
       </c>
     </row>
     <row r="103">
@@ -5340,7 +5321,7 @@
         <v>5</v>
       </c>
       <c r="D107" t="n">
-        <v>0.19896653835297</v>
+        <v>0.1989665383529699</v>
       </c>
     </row>
     <row r="108">
@@ -5420,7 +5401,7 @@
         <v>5.6</v>
       </c>
       <c r="D112" t="n">
-        <v>0.2086829309096993</v>
+        <v>0.2086829309096992</v>
       </c>
     </row>
     <row r="113">
@@ -5452,7 +5433,7 @@
         <v>5.1</v>
       </c>
       <c r="D114" t="n">
-        <v>0.1987019944069678</v>
+        <v>0.1987019944069677</v>
       </c>
     </row>
     <row r="115">
@@ -5468,7 +5449,7 @@
         <v>4.9</v>
       </c>
       <c r="D115" t="n">
-        <v>0.1940492012785181</v>
+        <v>0.194049201278518</v>
       </c>
     </row>
     <row r="116">
@@ -5612,7 +5593,7 @@
         <v>4.1</v>
       </c>
       <c r="D124" t="n">
-        <v>0.1944966162606</v>
+        <v>0.1944966162605999</v>
       </c>
     </row>
     <row r="125">
@@ -5644,7 +5625,7 @@
         <v>4.1</v>
       </c>
       <c r="D126" t="n">
-        <v>0.1961475664806731</v>
+        <v>0.196147566480673</v>
       </c>
     </row>
     <row r="127">
@@ -5724,7 +5705,7 @@
         <v>4.4</v>
       </c>
       <c r="D131" t="n">
-        <v>0.2073371391083059</v>
+        <v>0.2073371391083058</v>
       </c>
     </row>
     <row r="132">
@@ -5788,7 +5769,7 @@
         <v>5</v>
       </c>
       <c r="D135" t="n">
-        <v>0.2230346650151756</v>
+        <v>0.2230346650151755</v>
       </c>
     </row>
     <row r="136">
@@ -5852,7 +5833,7 @@
         <v>5.6</v>
       </c>
       <c r="D139" t="n">
-        <v>0.2255393188876454</v>
+        <v>0.2255393188876453</v>
       </c>
     </row>
     <row r="140">
@@ -5916,7 +5897,7 @@
         <v>5.9</v>
       </c>
       <c r="D143" t="n">
-        <v>0.2257120628881144</v>
+        <v>0.2257120628881143</v>
       </c>
     </row>
     <row r="144">
@@ -5932,7 +5913,7 @@
         <v>6.1</v>
       </c>
       <c r="D144" t="n">
-        <v>0.2282672486775731</v>
+        <v>0.228267248677573</v>
       </c>
     </row>
     <row r="145">
@@ -5964,7 +5945,7 @@
         <v>6.1</v>
       </c>
       <c r="D146" t="n">
-        <v>0.2298259181428325</v>
+        <v>0.2298259181428324</v>
       </c>
     </row>
     <row r="147">
@@ -5980,7 +5961,7 @@
         <v>6.2</v>
       </c>
       <c r="D147" t="n">
-        <v>0.2328904567233725</v>
+        <v>0.2328904567233724</v>
       </c>
     </row>
     <row r="148">
@@ -6076,7 +6057,7 @@
         <v>5.9</v>
       </c>
       <c r="D153" t="n">
-        <v>0.2265726951791928</v>
+        <v>0.2265726951791927</v>
       </c>
     </row>
     <row r="154">
@@ -6108,7 +6089,7 @@
         <v>5.6</v>
       </c>
       <c r="D155" t="n">
-        <v>0.2207881384697674</v>
+        <v>0.2207881384697673</v>
       </c>
     </row>
     <row r="156">
@@ -6124,7 +6105,7 @@
         <v>5.5</v>
       </c>
       <c r="D156" t="n">
-        <v>0.2253823067762058</v>
+        <v>0.2253823067762057</v>
       </c>
     </row>
     <row r="157">
@@ -6140,7 +6121,7 @@
         <v>5.5</v>
       </c>
       <c r="D157" t="n">
-        <v>0.2291800617182597</v>
+        <v>0.2291800617182596</v>
       </c>
     </row>
     <row r="158">
@@ -6156,7 +6137,7 @@
         <v>5.4</v>
       </c>
       <c r="D158" t="n">
-        <v>0.2309754226259297</v>
+        <v>0.2309754226259296</v>
       </c>
     </row>
     <row r="159">
@@ -6172,7 +6153,7 @@
         <v>5.5</v>
       </c>
       <c r="D159" t="n">
-        <v>0.2314148940180176</v>
+        <v>0.2314148940180175</v>
       </c>
     </row>
     <row r="160">
@@ -6380,7 +6361,7 @@
         <v>6.2</v>
       </c>
       <c r="D172" t="n">
-        <v>0.2426468029894171</v>
+        <v>0.242646802989417</v>
       </c>
     </row>
     <row r="173">
@@ -6412,7 +6393,7 @@
         <v>6.5</v>
       </c>
       <c r="D174" t="n">
-        <v>0.2433142716617252</v>
+        <v>0.2433142716617251</v>
       </c>
     </row>
     <row r="175">
@@ -6428,7 +6409,7 @@
         <v>6.8</v>
       </c>
       <c r="D175" t="n">
-        <v>0.2445324170963497</v>
+        <v>0.2445324170963496</v>
       </c>
     </row>
     <row r="176">
@@ -6444,7 +6425,7 @@
         <v>6.7</v>
       </c>
       <c r="D176" t="n">
-        <v>0.2458421710504727</v>
+        <v>0.2458421710504726</v>
       </c>
     </row>
     <row r="177">
@@ -6508,7 +6489,7 @@
         <v>6.9</v>
       </c>
       <c r="D180" t="n">
-        <v>0.2474092835719974</v>
+        <v>0.2473780901728729</v>
       </c>
     </row>
     <row r="181">
@@ -6518,29 +6499,13 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="C181" t="n">
         <v>7.2</v>
       </c>
       <c r="D181" t="n">
-        <v>0.2514723625654082</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="B182" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="C182" t="n">
-        <v>7</v>
-      </c>
-      <c r="D182" t="n">
-        <v>0.2483289996014</v>
+        <v>0.2513878650925042</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: update IDC to 202605 BCB release (Mar-2026)
IDC reaches 0.954 (vs 1.000 in Feb-2026); all three components retreated.
</commit_message>
<xml_diff>
--- a/data/processed/idc_data.xlsx
+++ b/data/processed/idc_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -847,13 +847,13 @@
         <v>0.2272727272727273</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D37" t="n">
         <v>0.8309695443551434</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3723552670132117</v>
+        <v>0.3723552670132118</v>
       </c>
     </row>
     <row r="38">
@@ -866,7 +866,7 @@
         <v>0.1818181818181812</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
@@ -885,7 +885,7 @@
         <v>0.1818181818181812</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
         <v>0.2727272727272735</v>
       </c>
       <c r="C41" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.3181818181818179</v>
+        <v>0.318181818181818</v>
       </c>
       <c r="C42" t="n">
         <v>0.1176470588235295</v>
@@ -948,7 +948,7 @@
         <v>0.8324983307105308</v>
       </c>
       <c r="E42" t="n">
-        <v>0.4227757359052927</v>
+        <v>0.4227757359052928</v>
       </c>
     </row>
     <row r="43">
@@ -999,7 +999,7 @@
         <v>0.2727272727272735</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D45" t="n">
         <v>0.7830522467498834</v>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.4090909090909085</v>
+        <v>0.4090909090909086</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -1059,10 +1059,10 @@
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4546540657780137</v>
+        <v>0.4546540657780138</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4242786279866108</v>
+        <v>0.4242786279866109</v>
       </c>
     </row>
     <row r="49">
@@ -1110,13 +1110,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.9545454545454556</v>
+        <v>0.9545454545454555</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0499999999999998</v>
+        <v>0.04999999999999982</v>
       </c>
       <c r="D51" t="n">
-        <v>0.9191340608899672</v>
+        <v>0.9191340608899673</v>
       </c>
       <c r="E51" t="n">
         <v>0.6412265051451409</v>
@@ -1129,10 +1129,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.9545454545454556</v>
+        <v>0.9545454545454555</v>
       </c>
       <c r="C52" t="n">
-        <v>0.1</v>
+        <v>0.1000000000000001</v>
       </c>
       <c r="D52" t="n">
         <v>0.9354739862101402</v>
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.9545454545454556</v>
+        <v>0.9545454545454555</v>
       </c>
       <c r="C53" t="n">
-        <v>0.0499999999999998</v>
+        <v>0.04999999999999982</v>
       </c>
       <c r="D53" t="n">
-        <v>0.9759592328097708</v>
+        <v>0.9759592328097707</v>
       </c>
       <c r="E53" t="n">
         <v>0.6601682291184087</v>
@@ -1170,7 +1170,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>0.1</v>
+        <v>0.1000000000000001</v>
       </c>
       <c r="D54" t="n">
         <v>0.8883007681125101</v>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.4400000000000005</v>
+        <v>0.4400000000000006</v>
       </c>
       <c r="C60" t="n">
         <v>0.5</v>
@@ -1325,7 +1325,7 @@
         <v>0.5</v>
       </c>
       <c r="D62" t="n">
-        <v>0.9725506805246664</v>
+        <v>0.9725506805246665</v>
       </c>
       <c r="E62" t="n">
         <v>0.6908502268415555</v>
@@ -1363,7 +1363,7 @@
         <v>0.5499999999999998</v>
       </c>
       <c r="D64" t="n">
-        <v>0.97499432097947</v>
+        <v>0.9749943209794701</v>
       </c>
       <c r="E64" t="n">
         <v>0.7349981069931566</v>
@@ -1382,7 +1382,7 @@
         <v>0.5</v>
       </c>
       <c r="D65" t="n">
-        <v>0.9310890047696612</v>
+        <v>0.9310890047696613</v>
       </c>
       <c r="E65" t="n">
         <v>0.7170296682565538</v>
@@ -1499,7 +1499,7 @@
         <v>0.1978798745881518</v>
       </c>
       <c r="E71" t="n">
-        <v>0.3326266248627172</v>
+        <v>0.3326266248627173</v>
       </c>
     </row>
     <row r="72">
@@ -1556,7 +1556,7 @@
         <v>0.3628231483643701</v>
       </c>
       <c r="E74" t="n">
-        <v>0.3309410494547899</v>
+        <v>0.33094104945479</v>
       </c>
     </row>
     <row r="75">
@@ -1566,13 +1566,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.1200000000000002</v>
+        <v>0.1200000000000003</v>
       </c>
       <c r="C75" t="n">
         <v>0.2999999999999998</v>
       </c>
       <c r="D75" t="n">
-        <v>0.4356421767454645</v>
+        <v>0.4356421767454646</v>
       </c>
       <c r="E75" t="n">
         <v>0.2852140589151549</v>
@@ -1629,10 +1629,10 @@
         <v>0.25</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2399283557599175</v>
+        <v>0.2399283557599176</v>
       </c>
       <c r="E78" t="n">
-        <v>0.2003464889570096</v>
+        <v>0.2003464889570097</v>
       </c>
     </row>
     <row r="79">
@@ -1648,7 +1648,7 @@
         <v>0.25</v>
       </c>
       <c r="D79" t="n">
-        <v>0.1629527256875272</v>
+        <v>0.1629527256875273</v>
       </c>
       <c r="E79" t="n">
         <v>0.2117249826365829</v>
@@ -1670,7 +1670,7 @@
         <v>0.1102481552651509</v>
       </c>
       <c r="E80" t="n">
-        <v>0.2021814838538157</v>
+        <v>0.2021814838538158</v>
       </c>
     </row>
     <row r="81">
@@ -1702,7 +1702,7 @@
         <v>0.1111111111111114</v>
       </c>
       <c r="C82" t="n">
-        <v>0.1</v>
+        <v>0.1000000000000001</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.0370370370370362</v>
+        <v>0.03703703703703626</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
@@ -1727,7 +1727,7 @@
         <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>0.0123456790123454</v>
+        <v>0.01234567901234542</v>
       </c>
     </row>
     <row r="84">
@@ -1743,10 +1743,10 @@
         <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>0.07217268456268749</v>
+        <v>0.07217268456268752</v>
       </c>
       <c r="E84" t="n">
-        <v>0.0240575615208958</v>
+        <v>0.02405756152089584</v>
       </c>
     </row>
     <row r="85">
@@ -1765,7 +1765,7 @@
         <v>0.2373397296057668</v>
       </c>
       <c r="E85" t="n">
-        <v>0.0791132432019222</v>
+        <v>0.07911324320192227</v>
       </c>
     </row>
     <row r="86">
@@ -1775,16 +1775,16 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.0357142857142862</v>
+        <v>0.03571428571428621</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
       </c>
       <c r="D86" t="n">
-        <v>0.1736702105847081</v>
+        <v>0.1736702105847082</v>
       </c>
       <c r="E86" t="n">
-        <v>0.06979483209966469</v>
+        <v>0.06979483209966479</v>
       </c>
     </row>
     <row r="87">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.1428571428571435</v>
+        <v>0.1428571428571436</v>
       </c>
       <c r="C87" t="n">
         <v>0</v>
@@ -1819,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="D88" t="n">
-        <v>0.1512087838932728</v>
+        <v>0.1512087838932729</v>
       </c>
       <c r="E88" t="n">
         <v>0.1337362612977575</v>
@@ -1838,10 +1838,10 @@
         <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>0.1751051323246209</v>
+        <v>0.175105132324621</v>
       </c>
       <c r="E89" t="n">
-        <v>0.1655112345843976</v>
+        <v>0.1655112345843977</v>
       </c>
     </row>
     <row r="90">
@@ -1854,13 +1854,13 @@
         <v>0.2142857142857147</v>
       </c>
       <c r="C90" t="n">
-        <v>0.043478260869565</v>
+        <v>0.04347826086956506</v>
       </c>
       <c r="D90" t="n">
-        <v>0.09045990357805481</v>
+        <v>0.09045990357805485</v>
       </c>
       <c r="E90" t="n">
-        <v>0.1160746262444448</v>
+        <v>0.1160746262444449</v>
       </c>
     </row>
     <row r="91">
@@ -1870,16 +1870,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.1071428571428573</v>
+        <v>0.1071428571428574</v>
       </c>
       <c r="C91" t="n">
-        <v>0.043478260869565</v>
+        <v>0.04347826086956506</v>
       </c>
       <c r="D91" t="n">
-        <v>0.0383129816107087</v>
+        <v>0.03831298161070876</v>
       </c>
       <c r="E91" t="n">
-        <v>0.06297803320771039</v>
+        <v>0.06297803320771041</v>
       </c>
     </row>
     <row r="92">
@@ -1889,16 +1889,16 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.1428571428571435</v>
+        <v>0.1428571428571436</v>
       </c>
       <c r="C92" t="n">
         <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>0.0179106796724274</v>
+        <v>0.01791067967242742</v>
       </c>
       <c r="E92" t="n">
-        <v>0.0535892741765236</v>
+        <v>0.05358927417652367</v>
       </c>
     </row>
     <row r="93">
@@ -1908,16 +1908,16 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.1071428571428573</v>
+        <v>0.1071428571428574</v>
       </c>
       <c r="C93" t="n">
         <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>0.0489874235180162</v>
+        <v>0.04898742351801629</v>
       </c>
       <c r="E93" t="n">
-        <v>0.0520434268869578</v>
+        <v>0.05204342688695789</v>
       </c>
     </row>
     <row r="94">
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="D94" t="n">
-        <v>0.0061634902446653</v>
+        <v>0.006163490244665353</v>
       </c>
       <c r="E94" t="n">
-        <v>0.0615783062720312</v>
+        <v>0.06157830627203129</v>
       </c>
     </row>
     <row r="95">
@@ -1971,10 +1971,10 @@
         <v>0</v>
       </c>
       <c r="D96" t="n">
-        <v>0.123980471048117</v>
+        <v>0.1239804710481171</v>
       </c>
       <c r="E96" t="n">
-        <v>0.148469680825563</v>
+        <v>0.1484696808255631</v>
       </c>
     </row>
     <row r="97">
@@ -1990,7 +1990,7 @@
         <v>0</v>
       </c>
       <c r="D97" t="n">
-        <v>0.2448778821631854</v>
+        <v>0.2448778821631855</v>
       </c>
       <c r="E97" t="n">
         <v>0.2125783416734429</v>
@@ -2012,7 +2012,7 @@
         <v>0.2320166827458945</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2082912752010125</v>
+        <v>0.2082912752010126</v>
       </c>
     </row>
     <row r="99">
@@ -2028,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="D99" t="n">
-        <v>0.2854673416493078</v>
+        <v>0.2854673416493079</v>
       </c>
       <c r="E99" t="n">
         <v>0.2856319710259599</v>
@@ -2044,13 +2044,13 @@
         <v>0.6785714285714292</v>
       </c>
       <c r="C100" t="n">
-        <v>0.0399999999999998</v>
+        <v>0.03999999999999986</v>
       </c>
       <c r="D100" t="n">
         <v>0.2905293572727042</v>
       </c>
       <c r="E100" t="n">
-        <v>0.336366928614711</v>
+        <v>0.3363669286147111</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="C101" t="n">
-        <v>0.0399999999999998</v>
+        <v>0.03999999999999986</v>
       </c>
       <c r="D101" t="n">
         <v>0.3513175817075109</v>
@@ -2082,7 +2082,7 @@
         <v>0.8999999999999998</v>
       </c>
       <c r="C102" t="n">
-        <v>0.0399999999999998</v>
+        <v>0.03999999999999986</v>
       </c>
       <c r="D102" t="n">
         <v>0.2860368403049701</v>
@@ -2101,7 +2101,7 @@
         <v>0.9333333333333336</v>
       </c>
       <c r="C103" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="D103" t="n">
         <v>0.2805459391879865</v>
@@ -2123,7 +2123,7 @@
         <v>0.1199999999999999</v>
       </c>
       <c r="D104" t="n">
-        <v>0.2809435606936264</v>
+        <v>0.2809435606936265</v>
       </c>
       <c r="E104" t="n">
         <v>0.3558700757867643</v>
@@ -2164,7 +2164,7 @@
         <v>0.1981927225528276</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2393975741842757</v>
+        <v>0.2393975741842758</v>
       </c>
     </row>
     <row r="107">
@@ -2180,10 +2180,10 @@
         <v>0.1199999999999999</v>
       </c>
       <c r="D107" t="n">
-        <v>0.0247978497132711</v>
+        <v>0.02479784971327119</v>
       </c>
       <c r="E107" t="n">
-        <v>0.1371548387933126</v>
+        <v>0.1371548387933127</v>
       </c>
     </row>
     <row r="108">
@@ -2196,7 +2196,7 @@
         <v>0.2666666666666669</v>
       </c>
       <c r="C108" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="D108" t="n">
         <v>0.1035980211576326</v>
@@ -2215,10 +2215,10 @@
         <v>0.2333333333333331</v>
       </c>
       <c r="C109" t="n">
-        <v>0.1599999999999997</v>
+        <v>0.1599999999999998</v>
       </c>
       <c r="D109" t="n">
-        <v>0.2048299465559414</v>
+        <v>0.2048299465559415</v>
       </c>
       <c r="E109" t="n">
         <v>0.1993877599630914</v>
@@ -2253,13 +2253,13 @@
         <v>0.3999999999999997</v>
       </c>
       <c r="C111" t="n">
-        <v>0.3199999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="D111" t="n">
         <v>0.4283229775251577</v>
       </c>
       <c r="E111" t="n">
-        <v>0.3827743258417191</v>
+        <v>0.3827743258417192</v>
       </c>
     </row>
     <row r="112">
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>0.3599999999999997</v>
+        <v>0.3599999999999998</v>
       </c>
       <c r="D112" t="n">
-        <v>0.316575811270907</v>
+        <v>0.3165758112709071</v>
       </c>
       <c r="E112" t="n">
         <v>0.2255252704236356</v>
@@ -2291,13 +2291,13 @@
         <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0.2399999999999998</v>
+        <v>0.2399999999999999</v>
       </c>
       <c r="D113" t="n">
         <v>0.1678060787477241</v>
       </c>
       <c r="E113" t="n">
-        <v>0.1359353595825746</v>
+        <v>0.1359353595825747</v>
       </c>
     </row>
     <row r="114">
@@ -2310,13 +2310,13 @@
         <v>0</v>
       </c>
       <c r="C114" t="n">
-        <v>0.1599999999999997</v>
+        <v>0.1599999999999998</v>
       </c>
       <c r="D114" t="n">
-        <v>0.0168537395040272</v>
+        <v>0.01685373950402727</v>
       </c>
       <c r="E114" t="n">
-        <v>0.0589512465013423</v>
+        <v>0.05895124650134235</v>
       </c>
     </row>
     <row r="115">
@@ -2329,13 +2329,13 @@
         <v>0</v>
       </c>
       <c r="C115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
       </c>
       <c r="E115" t="n">
-        <v>0.0266666666666666</v>
+        <v>0.02666666666666669</v>
       </c>
     </row>
     <row r="116">
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.0588235294117641</v>
+        <v>0.05882352941176417</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="E116" t="n">
-        <v>0.0196078431372547</v>
+        <v>0.01960784313725472</v>
       </c>
     </row>
     <row r="117">
@@ -2373,7 +2373,7 @@
         <v>0</v>
       </c>
       <c r="E117" t="n">
-        <v>0.0588235294117646</v>
+        <v>0.05882352941176464</v>
       </c>
     </row>
     <row r="118">
@@ -2411,7 +2411,7 @@
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>0.1568627450980391</v>
+        <v>0.1568627450980392</v>
       </c>
     </row>
     <row r="120">
@@ -2468,7 +2468,7 @@
         <v>0.2153533575103212</v>
       </c>
       <c r="E122" t="n">
-        <v>0.2482550407387345</v>
+        <v>0.2482550407387346</v>
       </c>
     </row>
     <row r="123">
@@ -2500,7 +2500,7 @@
         <v>0.6078431372549018</v>
       </c>
       <c r="C124" t="n">
-        <v>0.0312499999999998</v>
+        <v>0.03124999999999989</v>
       </c>
       <c r="D124" t="n">
         <v>0.2545599775084994</v>
@@ -2525,7 +2525,7 @@
         <v>0.2814720600383868</v>
       </c>
       <c r="E125" t="n">
-        <v>0.3029743468101812</v>
+        <v>0.3029743468101813</v>
       </c>
     </row>
     <row r="126">
@@ -2538,7 +2538,7 @@
         <v>0.7058823529411763</v>
       </c>
       <c r="C126" t="n">
-        <v>0.0312499999999998</v>
+        <v>0.03124999999999989</v>
       </c>
       <c r="D126" t="n">
         <v>0.2878714351788128</v>
@@ -2557,7 +2557,7 @@
         <v>0.7843137254901964</v>
       </c>
       <c r="C127" t="n">
-        <v>0.0312499999999998</v>
+        <v>0.03124999999999989</v>
       </c>
       <c r="D127" t="n">
         <v>0.3567797887508668</v>
@@ -2573,16 +2573,16 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.9607843137254904</v>
+        <v>0.9607843137254903</v>
       </c>
       <c r="C128" t="n">
-        <v>0.0625</v>
+        <v>0.06250000000000006</v>
       </c>
       <c r="D128" t="n">
         <v>0.4338893293994195</v>
       </c>
       <c r="E128" t="n">
-        <v>0.4857245477083032</v>
+        <v>0.4857245477083033</v>
       </c>
     </row>
     <row r="129">
@@ -2595,7 +2595,7 @@
         <v>1</v>
       </c>
       <c r="C129" t="n">
-        <v>0.0625</v>
+        <v>0.06250000000000006</v>
       </c>
       <c r="D129" t="n">
         <v>0.5109885971651589</v>
@@ -2614,7 +2614,7 @@
         <v>1</v>
       </c>
       <c r="C130" t="n">
-        <v>0.0937499999999999</v>
+        <v>0.09374999999999994</v>
       </c>
       <c r="D130" t="n">
         <v>0.5224447035496396</v>
@@ -2671,7 +2671,7 @@
         <v>0.9242424242424242</v>
       </c>
       <c r="C133" t="n">
-        <v>0.21875</v>
+        <v>0.2187500000000001</v>
       </c>
       <c r="D133" t="n">
         <v>0.7999634422509253</v>
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.9545454545454544</v>
+        <v>0.9545454545454545</v>
       </c>
       <c r="C137" t="n">
-        <v>0.375</v>
+        <v>0.3750000000000001</v>
       </c>
       <c r="D137" t="n">
         <v>0.8621984129111688</v>
@@ -2826,7 +2826,7 @@
         <v>0.5624999999999999</v>
       </c>
       <c r="D141" t="n">
-        <v>0.9434585701441284</v>
+        <v>0.9434585701441283</v>
       </c>
       <c r="E141" t="n">
         <v>0.8353195233813761</v>
@@ -2845,7 +2845,7 @@
         <v>0.5624999999999999</v>
       </c>
       <c r="D142" t="n">
-        <v>0.93410039035488</v>
+        <v>0.9341003903548799</v>
       </c>
       <c r="E142" t="n">
         <v>0.8322001301182933</v>
@@ -2883,7 +2883,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D144" t="n">
-        <v>0.9359548364085428</v>
+        <v>0.9359548364085427</v>
       </c>
       <c r="E144" t="n">
         <v>0.8640682788028475</v>
@@ -2921,7 +2921,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D146" t="n">
-        <v>0.9534504164253912</v>
+        <v>0.9534504164253911</v>
       </c>
       <c r="E146" t="n">
         <v>0.8699001388084637</v>
@@ -2962,7 +2962,7 @@
         <v>0.987505664722233</v>
       </c>
       <c r="E148" t="n">
-        <v>0.9020852215740776</v>
+        <v>0.9020852215740777</v>
       </c>
     </row>
     <row r="149">
@@ -3016,7 +3016,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D151" t="n">
-        <v>0.9045886593715888</v>
+        <v>0.9045886593715887</v>
       </c>
       <c r="E151" t="n">
         <v>0.8094361796298871</v>
@@ -3168,7 +3168,7 @@
         <v>0.46875</v>
       </c>
       <c r="D159" t="n">
-        <v>0.9710731241272008</v>
+        <v>0.9710731241272009</v>
       </c>
       <c r="E159" t="n">
         <v>0.7369691538255329</v>
@@ -3187,7 +3187,7 @@
         <v>0.46875</v>
       </c>
       <c r="D160" t="n">
-        <v>0.9526198528080616</v>
+        <v>0.9526198528080617</v>
       </c>
       <c r="E160" t="n">
         <v>0.7308180633858198</v>
@@ -3206,7 +3206,7 @@
         <v>0.4375000000000001</v>
       </c>
       <c r="D161" t="n">
-        <v>0.9347747781531665</v>
+        <v>0.9347747781531663</v>
       </c>
       <c r="E161" t="n">
         <v>0.7265012312719391</v>
@@ -3225,7 +3225,7 @@
         <v>0.46875</v>
       </c>
       <c r="D162" t="n">
-        <v>0.9185303003362744</v>
+        <v>0.9185303003362743</v>
       </c>
       <c r="E162" t="n">
         <v>0.7395352005136978</v>
@@ -3244,7 +3244,7 @@
         <v>0.46875</v>
       </c>
       <c r="D163" t="n">
-        <v>0.9405333228759576</v>
+        <v>0.9405333228759577</v>
       </c>
       <c r="E163" t="n">
         <v>0.7589177341313434</v>
@@ -3263,7 +3263,7 @@
         <v>0.4999999999999999</v>
       </c>
       <c r="D164" t="n">
-        <v>0.982332204543228</v>
+        <v>0.9823322045432281</v>
       </c>
       <c r="E164" t="n">
         <v>0.7792512970967387</v>
@@ -3282,7 +3282,7 @@
         <v>0.4375000000000001</v>
       </c>
       <c r="D165" t="n">
-        <v>0.9844349745515916</v>
+        <v>0.9844349745515915</v>
       </c>
       <c r="E165" t="n">
         <v>0.7591188870995266</v>
@@ -3317,7 +3317,7 @@
         <v>0.8915662650602411</v>
       </c>
       <c r="C167" t="n">
-        <v>0.375</v>
+        <v>0.3750000000000001</v>
       </c>
       <c r="D167" t="n">
         <v>0.908477471644922</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.9156626506024096</v>
+        <v>0.9156626506024097</v>
       </c>
       <c r="C168" t="n">
         <v>0.4999999999999999</v>
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.9397590361445785</v>
+        <v>0.9397590361445783</v>
       </c>
       <c r="C171" t="n">
         <v>0.625</v>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.9638554216867472</v>
+        <v>0.9638554216867473</v>
       </c>
       <c r="C172" t="n">
         <v>0.6875</v>
@@ -3453,7 +3453,7 @@
         <v>0.78125</v>
       </c>
       <c r="D174" t="n">
-        <v>0.9940035084602724</v>
+        <v>0.9940035084602725</v>
       </c>
       <c r="E174" t="n">
         <v>0.9090202457919784</v>
@@ -3529,10 +3529,10 @@
         <v>0.84375</v>
       </c>
       <c r="D178" t="n">
-        <v>0.9929551033202064</v>
+        <v>0.9929551033202063</v>
       </c>
       <c r="E178" t="n">
-        <v>0.9346988025560108</v>
+        <v>0.9346988025560109</v>
       </c>
     </row>
     <row r="179">
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.9891304347826084</v>
+        <v>0.9891304347826085</v>
       </c>
       <c r="C179" t="n">
         <v>0.8749999999999999</v>
@@ -3564,13 +3564,13 @@
         <v>1</v>
       </c>
       <c r="C180" t="n">
-        <v>0.90625</v>
+        <v>0.9062500000000001</v>
       </c>
       <c r="D180" t="n">
-        <v>0.99175252624052</v>
+        <v>0.9922248499806769</v>
       </c>
       <c r="E180" t="n">
-        <v>0.9660008420801732</v>
+        <v>0.9661582833268924</v>
       </c>
     </row>
     <row r="181">
@@ -3590,6 +3590,25 @@
       </c>
       <c r="E181" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>0.9684210526315788</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0.954831548220203</v>
+      </c>
+      <c r="E182" t="n">
+        <v>0.9535842002839273</v>
       </c>
     </row>
   </sheetData>
@@ -3603,7 +3622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3641,7 +3660,7 @@
         <v>5.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2144837064952338</v>
+        <v>0.2144837064952339</v>
       </c>
     </row>
     <row r="3">
@@ -3657,7 +3676,7 @@
         <v>5.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2163189319384209</v>
+        <v>0.216318931938421</v>
       </c>
     </row>
     <row r="4">
@@ -3689,7 +3708,7 @@
         <v>5.9</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2158826655184727</v>
+        <v>0.2158826655184728</v>
       </c>
     </row>
     <row r="6">
@@ -3753,7 +3772,7 @@
         <v>6.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2179910005812396</v>
+        <v>0.2179910005812397</v>
       </c>
     </row>
     <row r="10">
@@ -3769,7 +3788,7 @@
         <v>6.6</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2182622171978538</v>
+        <v>0.2182622171978539</v>
       </c>
     </row>
     <row r="11">
@@ -3785,7 +3804,7 @@
         <v>6.7</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2133141087974605</v>
+        <v>0.2133141087974606</v>
       </c>
     </row>
     <row r="12">
@@ -3849,7 +3868,7 @@
         <v>7.1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2221233325942453</v>
+        <v>0.2221233325942454</v>
       </c>
     </row>
     <row r="16">
@@ -3865,7 +3884,7 @@
         <v>7.2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2207697538835359</v>
+        <v>0.220769753883536</v>
       </c>
     </row>
     <row r="17">
@@ -3881,7 +3900,7 @@
         <v>7.1</v>
       </c>
       <c r="D17" t="n">
-        <v>0.2197200510871162</v>
+        <v>0.2197200510871163</v>
       </c>
     </row>
     <row r="18">
@@ -3897,7 +3916,7 @@
         <v>7.2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.2177195914744851</v>
+        <v>0.2177195914744852</v>
       </c>
     </row>
     <row r="19">
@@ -4025,7 +4044,7 @@
         <v>6.6</v>
       </c>
       <c r="D26" t="n">
-        <v>0.2181028585196966</v>
+        <v>0.2181028585196967</v>
       </c>
     </row>
     <row r="27">
@@ -4057,7 +4076,7 @@
         <v>6.6</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2172222433013913</v>
+        <v>0.2172222433013914</v>
       </c>
     </row>
     <row r="29">
@@ -4073,7 +4092,7 @@
         <v>6.3</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2178010163122743</v>
+        <v>0.2178010163122744</v>
       </c>
     </row>
     <row r="30">
@@ -4105,7 +4124,7 @@
         <v>6.1</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2167167319171493</v>
+        <v>0.2167167319171494</v>
       </c>
     </row>
     <row r="32">
@@ -4153,7 +4172,7 @@
         <v>5.7</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2187602876319877</v>
+        <v>0.2187602876319878</v>
       </c>
     </row>
     <row r="35">
@@ -4201,7 +4220,7 @@
         <v>5.6</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2202994011171442</v>
+        <v>0.2202994011171443</v>
       </c>
     </row>
     <row r="38">
@@ -4217,7 +4236,7 @@
         <v>5.6</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2224782495762382</v>
+        <v>0.2224782495762383</v>
       </c>
     </row>
     <row r="39">
@@ -4233,7 +4252,7 @@
         <v>5.6</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2254332403816361</v>
+        <v>0.2254332403816362</v>
       </c>
     </row>
     <row r="40">
@@ -4249,7 +4268,7 @@
         <v>5.7</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2249205544331555</v>
+        <v>0.2249205544331556</v>
       </c>
     </row>
     <row r="41">
@@ -4265,7 +4284,7 @@
         <v>5.6</v>
       </c>
       <c r="D41" t="n">
-        <v>0.2274453362709763</v>
+        <v>0.2274453362709764</v>
       </c>
     </row>
     <row r="42">
@@ -4281,7 +4300,7 @@
         <v>5.7</v>
       </c>
       <c r="D42" t="n">
-        <v>0.224746456738706</v>
+        <v>0.2247464567387061</v>
       </c>
     </row>
     <row r="43">
@@ -4297,7 +4316,7 @@
         <v>5.7</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2248368217595581</v>
+        <v>0.2248368217595582</v>
       </c>
     </row>
     <row r="44">
@@ -4313,7 +4332,7 @@
         <v>5.7</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2254800353761996</v>
+        <v>0.2254800353761997</v>
       </c>
     </row>
     <row r="45">
@@ -4377,7 +4396,7 @@
         <v>5.3</v>
       </c>
       <c r="D48" t="n">
-        <v>0.2186584209756128</v>
+        <v>0.2186584209756129</v>
       </c>
     </row>
     <row r="49">
@@ -4441,7 +4460,7 @@
         <v>5.4</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2264056574507283</v>
+        <v>0.2264056574507284</v>
       </c>
     </row>
     <row r="53">
@@ -4537,7 +4556,7 @@
         <v>6</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2285970857885172</v>
+        <v>0.2285970857885173</v>
       </c>
     </row>
     <row r="59">
@@ -4713,7 +4732,7 @@
         <v>6.2</v>
       </c>
       <c r="D69" t="n">
-        <v>0.2277393789965919</v>
+        <v>0.227739378996592</v>
       </c>
     </row>
     <row r="70">
@@ -4793,7 +4812,7 @@
         <v>5.9</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2186286523599864</v>
+        <v>0.2186286523599865</v>
       </c>
     </row>
     <row r="75">
@@ -4825,7 +4844,7 @@
         <v>5.9</v>
       </c>
       <c r="D76" t="n">
-        <v>0.2191753307115641</v>
+        <v>0.2191753307115642</v>
       </c>
     </row>
     <row r="77">
@@ -4841,7 +4860,7 @@
         <v>5.7</v>
       </c>
       <c r="D77" t="n">
-        <v>0.2175911308009367</v>
+        <v>0.2175911308009368</v>
       </c>
     </row>
     <row r="78">
@@ -4857,7 +4876,7 @@
         <v>5.7</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2161574089217934</v>
+        <v>0.2161574089217935</v>
       </c>
     </row>
     <row r="79">
@@ -4873,7 +4892,7 @@
         <v>5.7</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2146095360080124</v>
+        <v>0.2146095360080125</v>
       </c>
     </row>
     <row r="80">
@@ -4889,7 +4908,7 @@
         <v>5.6</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2135497203635995</v>
+        <v>0.2135497203635996</v>
       </c>
     </row>
     <row r="81">
@@ -4937,7 +4956,7 @@
         <v>5.2</v>
       </c>
       <c r="D83" t="n">
-        <v>0.2027358661530097</v>
+        <v>0.2027358661530098</v>
       </c>
     </row>
     <row r="84">
@@ -4953,7 +4972,7 @@
         <v>5.2</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2048076210931713</v>
+        <v>0.2048076210931714</v>
       </c>
     </row>
     <row r="85">
@@ -5001,7 +5020,7 @@
         <v>5.1</v>
       </c>
       <c r="D87" t="n">
-        <v>0.2087065635519887</v>
+        <v>0.2087065635519888</v>
       </c>
     </row>
     <row r="88">
@@ -5017,7 +5036,7 @@
         <v>5</v>
       </c>
       <c r="D88" t="n">
-        <v>0.2070763939707691</v>
+        <v>0.2070763939707692</v>
       </c>
     </row>
     <row r="89">
@@ -5081,7 +5100,7 @@
         <v>4.9</v>
       </c>
       <c r="D92" t="n">
-        <v>0.2032500016506407</v>
+        <v>0.2032500016506408</v>
       </c>
     </row>
     <row r="93">
@@ -5097,7 +5116,7 @@
         <v>4.9</v>
       </c>
       <c r="D93" t="n">
-        <v>0.2041420759579268</v>
+        <v>0.2041420759579269</v>
       </c>
     </row>
     <row r="94">
@@ -5113,7 +5132,7 @@
         <v>4.8</v>
       </c>
       <c r="D94" t="n">
-        <v>0.2029127923881968</v>
+        <v>0.2029127923881969</v>
       </c>
     </row>
     <row r="95">
@@ -5177,7 +5196,7 @@
         <v>4.7</v>
       </c>
       <c r="D98" t="n">
-        <v>0.205867057899216</v>
+        <v>0.2058670578992161</v>
       </c>
     </row>
     <row r="99">
@@ -5241,7 +5260,7 @@
         <v>4.8</v>
       </c>
       <c r="D102" t="n">
-        <v>0.2076659636631</v>
+        <v>0.2076659636631001</v>
       </c>
     </row>
     <row r="103">
@@ -5321,7 +5340,7 @@
         <v>5</v>
       </c>
       <c r="D107" t="n">
-        <v>0.1989665383529699</v>
+        <v>0.19896653835297</v>
       </c>
     </row>
     <row r="108">
@@ -5401,7 +5420,7 @@
         <v>5.6</v>
       </c>
       <c r="D112" t="n">
-        <v>0.2086829309096992</v>
+        <v>0.2086829309096993</v>
       </c>
     </row>
     <row r="113">
@@ -5433,7 +5452,7 @@
         <v>5.1</v>
       </c>
       <c r="D114" t="n">
-        <v>0.1987019944069677</v>
+        <v>0.1987019944069678</v>
       </c>
     </row>
     <row r="115">
@@ -5449,7 +5468,7 @@
         <v>4.9</v>
       </c>
       <c r="D115" t="n">
-        <v>0.194049201278518</v>
+        <v>0.1940492012785181</v>
       </c>
     </row>
     <row r="116">
@@ -5593,7 +5612,7 @@
         <v>4.1</v>
       </c>
       <c r="D124" t="n">
-        <v>0.1944966162605999</v>
+        <v>0.1944966162606</v>
       </c>
     </row>
     <row r="125">
@@ -5625,7 +5644,7 @@
         <v>4.1</v>
       </c>
       <c r="D126" t="n">
-        <v>0.196147566480673</v>
+        <v>0.1961475664806731</v>
       </c>
     </row>
     <row r="127">
@@ -5705,7 +5724,7 @@
         <v>4.4</v>
       </c>
       <c r="D131" t="n">
-        <v>0.2073371391083058</v>
+        <v>0.2073371391083059</v>
       </c>
     </row>
     <row r="132">
@@ -5769,7 +5788,7 @@
         <v>5</v>
       </c>
       <c r="D135" t="n">
-        <v>0.2230346650151755</v>
+        <v>0.2230346650151756</v>
       </c>
     </row>
     <row r="136">
@@ -5833,7 +5852,7 @@
         <v>5.6</v>
       </c>
       <c r="D139" t="n">
-        <v>0.2255393188876453</v>
+        <v>0.2255393188876454</v>
       </c>
     </row>
     <row r="140">
@@ -5897,7 +5916,7 @@
         <v>5.9</v>
       </c>
       <c r="D143" t="n">
-        <v>0.2257120628881143</v>
+        <v>0.2257120628881144</v>
       </c>
     </row>
     <row r="144">
@@ -5913,7 +5932,7 @@
         <v>6.1</v>
       </c>
       <c r="D144" t="n">
-        <v>0.228267248677573</v>
+        <v>0.2282672486775731</v>
       </c>
     </row>
     <row r="145">
@@ -5945,7 +5964,7 @@
         <v>6.1</v>
       </c>
       <c r="D146" t="n">
-        <v>0.2298259181428324</v>
+        <v>0.2298259181428325</v>
       </c>
     </row>
     <row r="147">
@@ -5961,7 +5980,7 @@
         <v>6.2</v>
       </c>
       <c r="D147" t="n">
-        <v>0.2328904567233724</v>
+        <v>0.2328904567233725</v>
       </c>
     </row>
     <row r="148">
@@ -6057,7 +6076,7 @@
         <v>5.9</v>
       </c>
       <c r="D153" t="n">
-        <v>0.2265726951791927</v>
+        <v>0.2265726951791928</v>
       </c>
     </row>
     <row r="154">
@@ -6089,7 +6108,7 @@
         <v>5.6</v>
       </c>
       <c r="D155" t="n">
-        <v>0.2207881384697673</v>
+        <v>0.2207881384697674</v>
       </c>
     </row>
     <row r="156">
@@ -6105,7 +6124,7 @@
         <v>5.5</v>
       </c>
       <c r="D156" t="n">
-        <v>0.2253823067762057</v>
+        <v>0.2253823067762058</v>
       </c>
     </row>
     <row r="157">
@@ -6121,7 +6140,7 @@
         <v>5.5</v>
       </c>
       <c r="D157" t="n">
-        <v>0.2291800617182596</v>
+        <v>0.2291800617182597</v>
       </c>
     </row>
     <row r="158">
@@ -6137,7 +6156,7 @@
         <v>5.4</v>
       </c>
       <c r="D158" t="n">
-        <v>0.2309754226259296</v>
+        <v>0.2309754226259297</v>
       </c>
     </row>
     <row r="159">
@@ -6153,7 +6172,7 @@
         <v>5.5</v>
       </c>
       <c r="D159" t="n">
-        <v>0.2314148940180175</v>
+        <v>0.2314148940180176</v>
       </c>
     </row>
     <row r="160">
@@ -6361,7 +6380,7 @@
         <v>6.2</v>
       </c>
       <c r="D172" t="n">
-        <v>0.242646802989417</v>
+        <v>0.2426468029894171</v>
       </c>
     </row>
     <row r="173">
@@ -6393,7 +6412,7 @@
         <v>6.5</v>
       </c>
       <c r="D174" t="n">
-        <v>0.2433142716617251</v>
+        <v>0.2433142716617252</v>
       </c>
     </row>
     <row r="175">
@@ -6409,7 +6428,7 @@
         <v>6.8</v>
       </c>
       <c r="D175" t="n">
-        <v>0.2445324170963496</v>
+        <v>0.2445324170963497</v>
       </c>
     </row>
     <row r="176">
@@ -6425,7 +6444,7 @@
         <v>6.7</v>
       </c>
       <c r="D176" t="n">
-        <v>0.2458421710504726</v>
+        <v>0.2458421710504727</v>
       </c>
     </row>
     <row r="177">
@@ -6489,7 +6508,7 @@
         <v>6.9</v>
       </c>
       <c r="D180" t="n">
-        <v>0.2473780901728729</v>
+        <v>0.2474092835719974</v>
       </c>
     </row>
     <row r="181">
@@ -6499,13 +6518,29 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>29.7</v>
+        <v>29.6</v>
       </c>
       <c r="C181" t="n">
         <v>7.2</v>
       </c>
       <c r="D181" t="n">
-        <v>0.2513878650925042</v>
+        <v>0.2514723625654082</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="C182" t="n">
+        <v>7</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0.2483289996014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: update IDC to 202605 BCB release
Update IDC data and report to the 202605 BCB release.

Includes the monthly raw release files, processed outputs, regenerated figures, the compiled report, and versioned monthly report pipeline/template rules so future updates preserve the agreed editorial and layout adjustments.
</commit_message>
<xml_diff>
--- a/data/processed/idc_data.xlsx
+++ b/data/processed/idc_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -847,13 +847,13 @@
         <v>0.2272727272727273</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D37" t="n">
         <v>0.8309695443551434</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3723552670132117</v>
+        <v>0.3723552670132118</v>
       </c>
     </row>
     <row r="38">
@@ -866,7 +866,7 @@
         <v>0.1818181818181812</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
@@ -885,7 +885,7 @@
         <v>0.1818181818181812</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
         <v>0.2727272727272735</v>
       </c>
       <c r="C41" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.3181818181818179</v>
+        <v>0.318181818181818</v>
       </c>
       <c r="C42" t="n">
         <v>0.1176470588235295</v>
@@ -948,7 +948,7 @@
         <v>0.8324983307105308</v>
       </c>
       <c r="E42" t="n">
-        <v>0.4227757359052927</v>
+        <v>0.4227757359052928</v>
       </c>
     </row>
     <row r="43">
@@ -999,7 +999,7 @@
         <v>0.2727272727272735</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0588235294117644</v>
+        <v>0.05882352941176449</v>
       </c>
       <c r="D45" t="n">
         <v>0.7830522467498834</v>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.4090909090909085</v>
+        <v>0.4090909090909086</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -1059,10 +1059,10 @@
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4546540657780137</v>
+        <v>0.4546540657780138</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4242786279866108</v>
+        <v>0.4242786279866109</v>
       </c>
     </row>
     <row r="49">
@@ -1110,13 +1110,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.9545454545454556</v>
+        <v>0.9545454545454555</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0499999999999998</v>
+        <v>0.04999999999999982</v>
       </c>
       <c r="D51" t="n">
-        <v>0.9191340608899672</v>
+        <v>0.9191340608899673</v>
       </c>
       <c r="E51" t="n">
         <v>0.6412265051451409</v>
@@ -1129,10 +1129,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.9545454545454556</v>
+        <v>0.9545454545454555</v>
       </c>
       <c r="C52" t="n">
-        <v>0.1</v>
+        <v>0.1000000000000001</v>
       </c>
       <c r="D52" t="n">
         <v>0.9354739862101402</v>
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.9545454545454556</v>
+        <v>0.9545454545454555</v>
       </c>
       <c r="C53" t="n">
-        <v>0.0499999999999998</v>
+        <v>0.04999999999999982</v>
       </c>
       <c r="D53" t="n">
-        <v>0.9759592328097708</v>
+        <v>0.9759592328097707</v>
       </c>
       <c r="E53" t="n">
         <v>0.6601682291184087</v>
@@ -1170,7 +1170,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>0.1</v>
+        <v>0.1000000000000001</v>
       </c>
       <c r="D54" t="n">
         <v>0.8883007681125101</v>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.4400000000000005</v>
+        <v>0.4400000000000006</v>
       </c>
       <c r="C60" t="n">
         <v>0.5</v>
@@ -1325,7 +1325,7 @@
         <v>0.5</v>
       </c>
       <c r="D62" t="n">
-        <v>0.9725506805246664</v>
+        <v>0.9725506805246665</v>
       </c>
       <c r="E62" t="n">
         <v>0.6908502268415555</v>
@@ -1363,7 +1363,7 @@
         <v>0.5499999999999998</v>
       </c>
       <c r="D64" t="n">
-        <v>0.97499432097947</v>
+        <v>0.9749943209794701</v>
       </c>
       <c r="E64" t="n">
         <v>0.7349981069931566</v>
@@ -1382,7 +1382,7 @@
         <v>0.5</v>
       </c>
       <c r="D65" t="n">
-        <v>0.9310890047696612</v>
+        <v>0.9310890047696613</v>
       </c>
       <c r="E65" t="n">
         <v>0.7170296682565538</v>
@@ -1499,7 +1499,7 @@
         <v>0.1978798745881518</v>
       </c>
       <c r="E71" t="n">
-        <v>0.3326266248627172</v>
+        <v>0.3326266248627173</v>
       </c>
     </row>
     <row r="72">
@@ -1556,7 +1556,7 @@
         <v>0.3628231483643701</v>
       </c>
       <c r="E74" t="n">
-        <v>0.3309410494547899</v>
+        <v>0.33094104945479</v>
       </c>
     </row>
     <row r="75">
@@ -1566,13 +1566,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.1200000000000002</v>
+        <v>0.1200000000000003</v>
       </c>
       <c r="C75" t="n">
         <v>0.2999999999999998</v>
       </c>
       <c r="D75" t="n">
-        <v>0.4356421767454645</v>
+        <v>0.4356421767454646</v>
       </c>
       <c r="E75" t="n">
         <v>0.2852140589151549</v>
@@ -1629,10 +1629,10 @@
         <v>0.25</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2399283557599175</v>
+        <v>0.2399283557599176</v>
       </c>
       <c r="E78" t="n">
-        <v>0.2003464889570096</v>
+        <v>0.2003464889570097</v>
       </c>
     </row>
     <row r="79">
@@ -1648,7 +1648,7 @@
         <v>0.25</v>
       </c>
       <c r="D79" t="n">
-        <v>0.1629527256875272</v>
+        <v>0.1629527256875273</v>
       </c>
       <c r="E79" t="n">
         <v>0.2117249826365829</v>
@@ -1670,7 +1670,7 @@
         <v>0.1102481552651509</v>
       </c>
       <c r="E80" t="n">
-        <v>0.2021814838538157</v>
+        <v>0.2021814838538158</v>
       </c>
     </row>
     <row r="81">
@@ -1702,7 +1702,7 @@
         <v>0.1111111111111114</v>
       </c>
       <c r="C82" t="n">
-        <v>0.1</v>
+        <v>0.1000000000000001</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.0370370370370362</v>
+        <v>0.03703703703703626</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
@@ -1727,7 +1727,7 @@
         <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>0.0123456790123454</v>
+        <v>0.01234567901234542</v>
       </c>
     </row>
     <row r="84">
@@ -1743,10 +1743,10 @@
         <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>0.07217268456268749</v>
+        <v>0.07217268456268752</v>
       </c>
       <c r="E84" t="n">
-        <v>0.0240575615208958</v>
+        <v>0.02405756152089584</v>
       </c>
     </row>
     <row r="85">
@@ -1765,7 +1765,7 @@
         <v>0.2373397296057668</v>
       </c>
       <c r="E85" t="n">
-        <v>0.0791132432019222</v>
+        <v>0.07911324320192227</v>
       </c>
     </row>
     <row r="86">
@@ -1775,16 +1775,16 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.0357142857142862</v>
+        <v>0.03571428571428621</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
       </c>
       <c r="D86" t="n">
-        <v>0.1736702105847081</v>
+        <v>0.1736702105847082</v>
       </c>
       <c r="E86" t="n">
-        <v>0.06979483209966469</v>
+        <v>0.06979483209966479</v>
       </c>
     </row>
     <row r="87">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.1428571428571435</v>
+        <v>0.1428571428571436</v>
       </c>
       <c r="C87" t="n">
         <v>0</v>
@@ -1819,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="D88" t="n">
-        <v>0.1512087838932728</v>
+        <v>0.1512087838932729</v>
       </c>
       <c r="E88" t="n">
         <v>0.1337362612977575</v>
@@ -1838,10 +1838,10 @@
         <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>0.1751051323246209</v>
+        <v>0.175105132324621</v>
       </c>
       <c r="E89" t="n">
-        <v>0.1655112345843976</v>
+        <v>0.1655112345843977</v>
       </c>
     </row>
     <row r="90">
@@ -1854,13 +1854,13 @@
         <v>0.2142857142857147</v>
       </c>
       <c r="C90" t="n">
-        <v>0.043478260869565</v>
+        <v>0.04347826086956506</v>
       </c>
       <c r="D90" t="n">
-        <v>0.09045990357805481</v>
+        <v>0.09045990357805485</v>
       </c>
       <c r="E90" t="n">
-        <v>0.1160746262444448</v>
+        <v>0.1160746262444449</v>
       </c>
     </row>
     <row r="91">
@@ -1870,16 +1870,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.1071428571428573</v>
+        <v>0.1071428571428574</v>
       </c>
       <c r="C91" t="n">
-        <v>0.043478260869565</v>
+        <v>0.04347826086956506</v>
       </c>
       <c r="D91" t="n">
-        <v>0.0383129816107087</v>
+        <v>0.03831298161070876</v>
       </c>
       <c r="E91" t="n">
-        <v>0.06297803320771039</v>
+        <v>0.06297803320771041</v>
       </c>
     </row>
     <row r="92">
@@ -1889,16 +1889,16 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.1428571428571435</v>
+        <v>0.1428571428571436</v>
       </c>
       <c r="C92" t="n">
         <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>0.0179106796724274</v>
+        <v>0.01791067967242742</v>
       </c>
       <c r="E92" t="n">
-        <v>0.0535892741765236</v>
+        <v>0.05358927417652367</v>
       </c>
     </row>
     <row r="93">
@@ -1908,16 +1908,16 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.1071428571428573</v>
+        <v>0.1071428571428574</v>
       </c>
       <c r="C93" t="n">
         <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>0.0489874235180162</v>
+        <v>0.04898742351801629</v>
       </c>
       <c r="E93" t="n">
-        <v>0.0520434268869578</v>
+        <v>0.05204342688695789</v>
       </c>
     </row>
     <row r="94">
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="D94" t="n">
-        <v>0.0061634902446653</v>
+        <v>0.006163490244665353</v>
       </c>
       <c r="E94" t="n">
-        <v>0.0615783062720312</v>
+        <v>0.06157830627203129</v>
       </c>
     </row>
     <row r="95">
@@ -1971,10 +1971,10 @@
         <v>0</v>
       </c>
       <c r="D96" t="n">
-        <v>0.123980471048117</v>
+        <v>0.1239804710481171</v>
       </c>
       <c r="E96" t="n">
-        <v>0.148469680825563</v>
+        <v>0.1484696808255631</v>
       </c>
     </row>
     <row r="97">
@@ -1990,7 +1990,7 @@
         <v>0</v>
       </c>
       <c r="D97" t="n">
-        <v>0.2448778821631854</v>
+        <v>0.2448778821631855</v>
       </c>
       <c r="E97" t="n">
         <v>0.2125783416734429</v>
@@ -2012,7 +2012,7 @@
         <v>0.2320166827458945</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2082912752010125</v>
+        <v>0.2082912752010126</v>
       </c>
     </row>
     <row r="99">
@@ -2028,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="D99" t="n">
-        <v>0.2854673416493078</v>
+        <v>0.2854673416493079</v>
       </c>
       <c r="E99" t="n">
         <v>0.2856319710259599</v>
@@ -2044,13 +2044,13 @@
         <v>0.6785714285714292</v>
       </c>
       <c r="C100" t="n">
-        <v>0.0399999999999998</v>
+        <v>0.03999999999999986</v>
       </c>
       <c r="D100" t="n">
         <v>0.2905293572727042</v>
       </c>
       <c r="E100" t="n">
-        <v>0.336366928614711</v>
+        <v>0.3363669286147111</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="C101" t="n">
-        <v>0.0399999999999998</v>
+        <v>0.03999999999999986</v>
       </c>
       <c r="D101" t="n">
         <v>0.3513175817075109</v>
@@ -2082,7 +2082,7 @@
         <v>0.8999999999999998</v>
       </c>
       <c r="C102" t="n">
-        <v>0.0399999999999998</v>
+        <v>0.03999999999999986</v>
       </c>
       <c r="D102" t="n">
         <v>0.2860368403049701</v>
@@ -2101,7 +2101,7 @@
         <v>0.9333333333333336</v>
       </c>
       <c r="C103" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="D103" t="n">
         <v>0.2805459391879865</v>
@@ -2123,7 +2123,7 @@
         <v>0.1199999999999999</v>
       </c>
       <c r="D104" t="n">
-        <v>0.2809435606936264</v>
+        <v>0.2809435606936265</v>
       </c>
       <c r="E104" t="n">
         <v>0.3558700757867643</v>
@@ -2164,7 +2164,7 @@
         <v>0.1981927225528276</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2393975741842757</v>
+        <v>0.2393975741842758</v>
       </c>
     </row>
     <row r="107">
@@ -2180,10 +2180,10 @@
         <v>0.1199999999999999</v>
       </c>
       <c r="D107" t="n">
-        <v>0.0247978497132711</v>
+        <v>0.02479784971327119</v>
       </c>
       <c r="E107" t="n">
-        <v>0.1371548387933126</v>
+        <v>0.1371548387933127</v>
       </c>
     </row>
     <row r="108">
@@ -2196,7 +2196,7 @@
         <v>0.2666666666666669</v>
       </c>
       <c r="C108" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="D108" t="n">
         <v>0.1035980211576326</v>
@@ -2215,10 +2215,10 @@
         <v>0.2333333333333331</v>
       </c>
       <c r="C109" t="n">
-        <v>0.1599999999999997</v>
+        <v>0.1599999999999998</v>
       </c>
       <c r="D109" t="n">
-        <v>0.2048299465559414</v>
+        <v>0.2048299465559415</v>
       </c>
       <c r="E109" t="n">
         <v>0.1993877599630914</v>
@@ -2253,13 +2253,13 @@
         <v>0.3999999999999997</v>
       </c>
       <c r="C111" t="n">
-        <v>0.3199999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="D111" t="n">
         <v>0.4283229775251577</v>
       </c>
       <c r="E111" t="n">
-        <v>0.3827743258417191</v>
+        <v>0.3827743258417192</v>
       </c>
     </row>
     <row r="112">
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>0.3599999999999997</v>
+        <v>0.3599999999999998</v>
       </c>
       <c r="D112" t="n">
-        <v>0.316575811270907</v>
+        <v>0.3165758112709071</v>
       </c>
       <c r="E112" t="n">
         <v>0.2255252704236356</v>
@@ -2291,13 +2291,13 @@
         <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0.2399999999999998</v>
+        <v>0.2399999999999999</v>
       </c>
       <c r="D113" t="n">
         <v>0.1678060787477241</v>
       </c>
       <c r="E113" t="n">
-        <v>0.1359353595825746</v>
+        <v>0.1359353595825747</v>
       </c>
     </row>
     <row r="114">
@@ -2310,13 +2310,13 @@
         <v>0</v>
       </c>
       <c r="C114" t="n">
-        <v>0.1599999999999997</v>
+        <v>0.1599999999999998</v>
       </c>
       <c r="D114" t="n">
-        <v>0.0168537395040272</v>
+        <v>0.01685373950402727</v>
       </c>
       <c r="E114" t="n">
-        <v>0.0589512465013423</v>
+        <v>0.05895124650134235</v>
       </c>
     </row>
     <row r="115">
@@ -2329,13 +2329,13 @@
         <v>0</v>
       </c>
       <c r="C115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
       </c>
       <c r="E115" t="n">
-        <v>0.0266666666666666</v>
+        <v>0.02666666666666669</v>
       </c>
     </row>
     <row r="116">
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.0588235294117641</v>
+        <v>0.05882352941176417</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="E116" t="n">
-        <v>0.0196078431372547</v>
+        <v>0.01960784313725472</v>
       </c>
     </row>
     <row r="117">
@@ -2373,7 +2373,7 @@
         <v>0</v>
       </c>
       <c r="E117" t="n">
-        <v>0.0588235294117646</v>
+        <v>0.05882352941176464</v>
       </c>
     </row>
     <row r="118">
@@ -2411,7 +2411,7 @@
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>0.1568627450980391</v>
+        <v>0.1568627450980392</v>
       </c>
     </row>
     <row r="120">
@@ -2468,7 +2468,7 @@
         <v>0.2153533575103212</v>
       </c>
       <c r="E122" t="n">
-        <v>0.2482550407387345</v>
+        <v>0.2482550407387346</v>
       </c>
     </row>
     <row r="123">
@@ -2500,7 +2500,7 @@
         <v>0.6078431372549018</v>
       </c>
       <c r="C124" t="n">
-        <v>0.0312499999999998</v>
+        <v>0.03124999999999989</v>
       </c>
       <c r="D124" t="n">
         <v>0.2545599775084994</v>
@@ -2525,7 +2525,7 @@
         <v>0.2814720600383868</v>
       </c>
       <c r="E125" t="n">
-        <v>0.3029743468101812</v>
+        <v>0.3029743468101813</v>
       </c>
     </row>
     <row r="126">
@@ -2538,7 +2538,7 @@
         <v>0.7058823529411763</v>
       </c>
       <c r="C126" t="n">
-        <v>0.0312499999999998</v>
+        <v>0.03124999999999989</v>
       </c>
       <c r="D126" t="n">
         <v>0.2878714351788128</v>
@@ -2557,7 +2557,7 @@
         <v>0.7843137254901964</v>
       </c>
       <c r="C127" t="n">
-        <v>0.0312499999999998</v>
+        <v>0.03124999999999989</v>
       </c>
       <c r="D127" t="n">
         <v>0.3567797887508668</v>
@@ -2573,16 +2573,16 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.9607843137254904</v>
+        <v>0.9607843137254903</v>
       </c>
       <c r="C128" t="n">
-        <v>0.0625</v>
+        <v>0.06250000000000006</v>
       </c>
       <c r="D128" t="n">
         <v>0.4338893293994195</v>
       </c>
       <c r="E128" t="n">
-        <v>0.4857245477083032</v>
+        <v>0.4857245477083033</v>
       </c>
     </row>
     <row r="129">
@@ -2595,7 +2595,7 @@
         <v>1</v>
       </c>
       <c r="C129" t="n">
-        <v>0.0625</v>
+        <v>0.06250000000000006</v>
       </c>
       <c r="D129" t="n">
         <v>0.5109885971651589</v>
@@ -2614,7 +2614,7 @@
         <v>1</v>
       </c>
       <c r="C130" t="n">
-        <v>0.0937499999999999</v>
+        <v>0.09374999999999994</v>
       </c>
       <c r="D130" t="n">
         <v>0.5224447035496396</v>
@@ -2671,7 +2671,7 @@
         <v>0.9242424242424242</v>
       </c>
       <c r="C133" t="n">
-        <v>0.21875</v>
+        <v>0.2187500000000001</v>
       </c>
       <c r="D133" t="n">
         <v>0.7999634422509253</v>
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.9545454545454544</v>
+        <v>0.9545454545454545</v>
       </c>
       <c r="C137" t="n">
-        <v>0.375</v>
+        <v>0.3750000000000001</v>
       </c>
       <c r="D137" t="n">
         <v>0.8621984129111688</v>
@@ -2826,7 +2826,7 @@
         <v>0.5624999999999999</v>
       </c>
       <c r="D141" t="n">
-        <v>0.9434585701441284</v>
+        <v>0.9434585701441283</v>
       </c>
       <c r="E141" t="n">
         <v>0.8353195233813761</v>
@@ -2845,7 +2845,7 @@
         <v>0.5624999999999999</v>
       </c>
       <c r="D142" t="n">
-        <v>0.93410039035488</v>
+        <v>0.9341003903548799</v>
       </c>
       <c r="E142" t="n">
         <v>0.8322001301182933</v>
@@ -2883,7 +2883,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D144" t="n">
-        <v>0.9359548364085428</v>
+        <v>0.9359548364085427</v>
       </c>
       <c r="E144" t="n">
         <v>0.8640682788028475</v>
@@ -2921,7 +2921,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D146" t="n">
-        <v>0.9534504164253912</v>
+        <v>0.9534504164253911</v>
       </c>
       <c r="E146" t="n">
         <v>0.8699001388084637</v>
@@ -2962,7 +2962,7 @@
         <v>0.987505664722233</v>
       </c>
       <c r="E148" t="n">
-        <v>0.9020852215740776</v>
+        <v>0.9020852215740777</v>
       </c>
     </row>
     <row r="149">
@@ -3016,7 +3016,7 @@
         <v>0.6562499999999999</v>
       </c>
       <c r="D151" t="n">
-        <v>0.9045886593715888</v>
+        <v>0.9045886593715887</v>
       </c>
       <c r="E151" t="n">
         <v>0.8094361796298871</v>
@@ -3168,7 +3168,7 @@
         <v>0.46875</v>
       </c>
       <c r="D159" t="n">
-        <v>0.9710731241272008</v>
+        <v>0.9710731241272009</v>
       </c>
       <c r="E159" t="n">
         <v>0.7369691538255329</v>
@@ -3187,7 +3187,7 @@
         <v>0.46875</v>
       </c>
       <c r="D160" t="n">
-        <v>0.9526198528080616</v>
+        <v>0.9526198528080617</v>
       </c>
       <c r="E160" t="n">
         <v>0.7308180633858198</v>
@@ -3206,7 +3206,7 @@
         <v>0.4375000000000001</v>
       </c>
       <c r="D161" t="n">
-        <v>0.9347747781531665</v>
+        <v>0.9347747781531663</v>
       </c>
       <c r="E161" t="n">
         <v>0.7265012312719391</v>
@@ -3225,7 +3225,7 @@
         <v>0.46875</v>
       </c>
       <c r="D162" t="n">
-        <v>0.9185303003362744</v>
+        <v>0.9185303003362743</v>
       </c>
       <c r="E162" t="n">
         <v>0.7395352005136978</v>
@@ -3244,7 +3244,7 @@
         <v>0.46875</v>
       </c>
       <c r="D163" t="n">
-        <v>0.9405333228759576</v>
+        <v>0.9405333228759577</v>
       </c>
       <c r="E163" t="n">
         <v>0.7589177341313434</v>
@@ -3263,7 +3263,7 @@
         <v>0.4999999999999999</v>
       </c>
       <c r="D164" t="n">
-        <v>0.982332204543228</v>
+        <v>0.9823322045432281</v>
       </c>
       <c r="E164" t="n">
         <v>0.7792512970967387</v>
@@ -3282,7 +3282,7 @@
         <v>0.4375000000000001</v>
       </c>
       <c r="D165" t="n">
-        <v>0.9844349745515916</v>
+        <v>0.9844349745515915</v>
       </c>
       <c r="E165" t="n">
         <v>0.7591188870995266</v>
@@ -3317,7 +3317,7 @@
         <v>0.8915662650602411</v>
       </c>
       <c r="C167" t="n">
-        <v>0.375</v>
+        <v>0.3750000000000001</v>
       </c>
       <c r="D167" t="n">
         <v>0.908477471644922</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.9156626506024096</v>
+        <v>0.9156626506024097</v>
       </c>
       <c r="C168" t="n">
         <v>0.4999999999999999</v>
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.9397590361445785</v>
+        <v>0.9397590361445783</v>
       </c>
       <c r="C171" t="n">
         <v>0.625</v>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.9638554216867472</v>
+        <v>0.9638554216867473</v>
       </c>
       <c r="C172" t="n">
         <v>0.6875</v>
@@ -3453,7 +3453,7 @@
         <v>0.78125</v>
       </c>
       <c r="D174" t="n">
-        <v>0.9940035084602724</v>
+        <v>0.9940035084602725</v>
       </c>
       <c r="E174" t="n">
         <v>0.9090202457919784</v>
@@ -3529,10 +3529,10 @@
         <v>0.84375</v>
       </c>
       <c r="D178" t="n">
-        <v>0.9929551033202064</v>
+        <v>0.9929551033202063</v>
       </c>
       <c r="E178" t="n">
-        <v>0.9346988025560108</v>
+        <v>0.9346988025560109</v>
       </c>
     </row>
     <row r="179">
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.9891304347826084</v>
+        <v>0.9891304347826085</v>
       </c>
       <c r="C179" t="n">
         <v>0.8749999999999999</v>
@@ -3564,13 +3564,13 @@
         <v>1</v>
       </c>
       <c r="C180" t="n">
-        <v>0.90625</v>
+        <v>0.9062500000000001</v>
       </c>
       <c r="D180" t="n">
-        <v>0.99175252624052</v>
+        <v>0.9922248499806769</v>
       </c>
       <c r="E180" t="n">
-        <v>0.9660008420801732</v>
+        <v>0.9661582833268924</v>
       </c>
     </row>
     <row r="181">
@@ -3590,6 +3590,25 @@
       </c>
       <c r="E181" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>0.9684210526315788</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0.954831548220203</v>
+      </c>
+      <c r="E182" t="n">
+        <v>0.9535842002839273</v>
       </c>
     </row>
   </sheetData>
@@ -3603,7 +3622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3641,7 +3660,7 @@
         <v>5.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2144837064952338</v>
+        <v>0.2144837064952339</v>
       </c>
     </row>
     <row r="3">
@@ -3657,7 +3676,7 @@
         <v>5.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2163189319384209</v>
+        <v>0.216318931938421</v>
       </c>
     </row>
     <row r="4">
@@ -3689,7 +3708,7 @@
         <v>5.9</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2158826655184727</v>
+        <v>0.2158826655184728</v>
       </c>
     </row>
     <row r="6">
@@ -3753,7 +3772,7 @@
         <v>6.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2179910005812396</v>
+        <v>0.2179910005812397</v>
       </c>
     </row>
     <row r="10">
@@ -3769,7 +3788,7 @@
         <v>6.6</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2182622171978538</v>
+        <v>0.2182622171978539</v>
       </c>
     </row>
     <row r="11">
@@ -3785,7 +3804,7 @@
         <v>6.7</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2133141087974605</v>
+        <v>0.2133141087974606</v>
       </c>
     </row>
     <row r="12">
@@ -3849,7 +3868,7 @@
         <v>7.1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2221233325942453</v>
+        <v>0.2221233325942454</v>
       </c>
     </row>
     <row r="16">
@@ -3865,7 +3884,7 @@
         <v>7.2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2207697538835359</v>
+        <v>0.220769753883536</v>
       </c>
     </row>
     <row r="17">
@@ -3881,7 +3900,7 @@
         <v>7.1</v>
       </c>
       <c r="D17" t="n">
-        <v>0.2197200510871162</v>
+        <v>0.2197200510871163</v>
       </c>
     </row>
     <row r="18">
@@ -3897,7 +3916,7 @@
         <v>7.2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.2177195914744851</v>
+        <v>0.2177195914744852</v>
       </c>
     </row>
     <row r="19">
@@ -4025,7 +4044,7 @@
         <v>6.6</v>
       </c>
       <c r="D26" t="n">
-        <v>0.2181028585196966</v>
+        <v>0.2181028585196967</v>
       </c>
     </row>
     <row r="27">
@@ -4057,7 +4076,7 @@
         <v>6.6</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2172222433013913</v>
+        <v>0.2172222433013914</v>
       </c>
     </row>
     <row r="29">
@@ -4073,7 +4092,7 @@
         <v>6.3</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2178010163122743</v>
+        <v>0.2178010163122744</v>
       </c>
     </row>
     <row r="30">
@@ -4105,7 +4124,7 @@
         <v>6.1</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2167167319171493</v>
+        <v>0.2167167319171494</v>
       </c>
     </row>
     <row r="32">
@@ -4153,7 +4172,7 @@
         <v>5.7</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2187602876319877</v>
+        <v>0.2187602876319878</v>
       </c>
     </row>
     <row r="35">
@@ -4201,7 +4220,7 @@
         <v>5.6</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2202994011171442</v>
+        <v>0.2202994011171443</v>
       </c>
     </row>
     <row r="38">
@@ -4217,7 +4236,7 @@
         <v>5.6</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2224782495762382</v>
+        <v>0.2224782495762383</v>
       </c>
     </row>
     <row r="39">
@@ -4233,7 +4252,7 @@
         <v>5.6</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2254332403816361</v>
+        <v>0.2254332403816362</v>
       </c>
     </row>
     <row r="40">
@@ -4249,7 +4268,7 @@
         <v>5.7</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2249205544331555</v>
+        <v>0.2249205544331556</v>
       </c>
     </row>
     <row r="41">
@@ -4265,7 +4284,7 @@
         <v>5.6</v>
       </c>
       <c r="D41" t="n">
-        <v>0.2274453362709763</v>
+        <v>0.2274453362709764</v>
       </c>
     </row>
     <row r="42">
@@ -4281,7 +4300,7 @@
         <v>5.7</v>
       </c>
       <c r="D42" t="n">
-        <v>0.224746456738706</v>
+        <v>0.2247464567387061</v>
       </c>
     </row>
     <row r="43">
@@ -4297,7 +4316,7 @@
         <v>5.7</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2248368217595581</v>
+        <v>0.2248368217595582</v>
       </c>
     </row>
     <row r="44">
@@ -4313,7 +4332,7 @@
         <v>5.7</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2254800353761996</v>
+        <v>0.2254800353761997</v>
       </c>
     </row>
     <row r="45">
@@ -4377,7 +4396,7 @@
         <v>5.3</v>
       </c>
       <c r="D48" t="n">
-        <v>0.2186584209756128</v>
+        <v>0.2186584209756129</v>
       </c>
     </row>
     <row r="49">
@@ -4441,7 +4460,7 @@
         <v>5.4</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2264056574507283</v>
+        <v>0.2264056574507284</v>
       </c>
     </row>
     <row r="53">
@@ -4537,7 +4556,7 @@
         <v>6</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2285970857885172</v>
+        <v>0.2285970857885173</v>
       </c>
     </row>
     <row r="59">
@@ -4713,7 +4732,7 @@
         <v>6.2</v>
       </c>
       <c r="D69" t="n">
-        <v>0.2277393789965919</v>
+        <v>0.227739378996592</v>
       </c>
     </row>
     <row r="70">
@@ -4793,7 +4812,7 @@
         <v>5.9</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2186286523599864</v>
+        <v>0.2186286523599865</v>
       </c>
     </row>
     <row r="75">
@@ -4825,7 +4844,7 @@
         <v>5.9</v>
       </c>
       <c r="D76" t="n">
-        <v>0.2191753307115641</v>
+        <v>0.2191753307115642</v>
       </c>
     </row>
     <row r="77">
@@ -4841,7 +4860,7 @@
         <v>5.7</v>
       </c>
       <c r="D77" t="n">
-        <v>0.2175911308009367</v>
+        <v>0.2175911308009368</v>
       </c>
     </row>
     <row r="78">
@@ -4857,7 +4876,7 @@
         <v>5.7</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2161574089217934</v>
+        <v>0.2161574089217935</v>
       </c>
     </row>
     <row r="79">
@@ -4873,7 +4892,7 @@
         <v>5.7</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2146095360080124</v>
+        <v>0.2146095360080125</v>
       </c>
     </row>
     <row r="80">
@@ -4889,7 +4908,7 @@
         <v>5.6</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2135497203635995</v>
+        <v>0.2135497203635996</v>
       </c>
     </row>
     <row r="81">
@@ -4937,7 +4956,7 @@
         <v>5.2</v>
       </c>
       <c r="D83" t="n">
-        <v>0.2027358661530097</v>
+        <v>0.2027358661530098</v>
       </c>
     </row>
     <row r="84">
@@ -4953,7 +4972,7 @@
         <v>5.2</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2048076210931713</v>
+        <v>0.2048076210931714</v>
       </c>
     </row>
     <row r="85">
@@ -5001,7 +5020,7 @@
         <v>5.1</v>
       </c>
       <c r="D87" t="n">
-        <v>0.2087065635519887</v>
+        <v>0.2087065635519888</v>
       </c>
     </row>
     <row r="88">
@@ -5017,7 +5036,7 @@
         <v>5</v>
       </c>
       <c r="D88" t="n">
-        <v>0.2070763939707691</v>
+        <v>0.2070763939707692</v>
       </c>
     </row>
     <row r="89">
@@ -5081,7 +5100,7 @@
         <v>4.9</v>
       </c>
       <c r="D92" t="n">
-        <v>0.2032500016506407</v>
+        <v>0.2032500016506408</v>
       </c>
     </row>
     <row r="93">
@@ -5097,7 +5116,7 @@
         <v>4.9</v>
       </c>
       <c r="D93" t="n">
-        <v>0.2041420759579268</v>
+        <v>0.2041420759579269</v>
       </c>
     </row>
     <row r="94">
@@ -5113,7 +5132,7 @@
         <v>4.8</v>
       </c>
       <c r="D94" t="n">
-        <v>0.2029127923881968</v>
+        <v>0.2029127923881969</v>
       </c>
     </row>
     <row r="95">
@@ -5177,7 +5196,7 @@
         <v>4.7</v>
       </c>
       <c r="D98" t="n">
-        <v>0.205867057899216</v>
+        <v>0.2058670578992161</v>
       </c>
     </row>
     <row r="99">
@@ -5241,7 +5260,7 @@
         <v>4.8</v>
       </c>
       <c r="D102" t="n">
-        <v>0.2076659636631</v>
+        <v>0.2076659636631001</v>
       </c>
     </row>
     <row r="103">
@@ -5321,7 +5340,7 @@
         <v>5</v>
       </c>
       <c r="D107" t="n">
-        <v>0.1989665383529699</v>
+        <v>0.19896653835297</v>
       </c>
     </row>
     <row r="108">
@@ -5401,7 +5420,7 @@
         <v>5.6</v>
       </c>
       <c r="D112" t="n">
-        <v>0.2086829309096992</v>
+        <v>0.2086829309096993</v>
       </c>
     </row>
     <row r="113">
@@ -5433,7 +5452,7 @@
         <v>5.1</v>
       </c>
       <c r="D114" t="n">
-        <v>0.1987019944069677</v>
+        <v>0.1987019944069678</v>
       </c>
     </row>
     <row r="115">
@@ -5449,7 +5468,7 @@
         <v>4.9</v>
       </c>
       <c r="D115" t="n">
-        <v>0.194049201278518</v>
+        <v>0.1940492012785181</v>
       </c>
     </row>
     <row r="116">
@@ -5593,7 +5612,7 @@
         <v>4.1</v>
       </c>
       <c r="D124" t="n">
-        <v>0.1944966162605999</v>
+        <v>0.1944966162606</v>
       </c>
     </row>
     <row r="125">
@@ -5625,7 +5644,7 @@
         <v>4.1</v>
       </c>
       <c r="D126" t="n">
-        <v>0.196147566480673</v>
+        <v>0.1961475664806731</v>
       </c>
     </row>
     <row r="127">
@@ -5705,7 +5724,7 @@
         <v>4.4</v>
       </c>
       <c r="D131" t="n">
-        <v>0.2073371391083058</v>
+        <v>0.2073371391083059</v>
       </c>
     </row>
     <row r="132">
@@ -5769,7 +5788,7 @@
         <v>5</v>
       </c>
       <c r="D135" t="n">
-        <v>0.2230346650151755</v>
+        <v>0.2230346650151756</v>
       </c>
     </row>
     <row r="136">
@@ -5833,7 +5852,7 @@
         <v>5.6</v>
       </c>
       <c r="D139" t="n">
-        <v>0.2255393188876453</v>
+        <v>0.2255393188876454</v>
       </c>
     </row>
     <row r="140">
@@ -5897,7 +5916,7 @@
         <v>5.9</v>
       </c>
       <c r="D143" t="n">
-        <v>0.2257120628881143</v>
+        <v>0.2257120628881144</v>
       </c>
     </row>
     <row r="144">
@@ -5913,7 +5932,7 @@
         <v>6.1</v>
       </c>
       <c r="D144" t="n">
-        <v>0.228267248677573</v>
+        <v>0.2282672486775731</v>
       </c>
     </row>
     <row r="145">
@@ -5945,7 +5964,7 @@
         <v>6.1</v>
       </c>
       <c r="D146" t="n">
-        <v>0.2298259181428324</v>
+        <v>0.2298259181428325</v>
       </c>
     </row>
     <row r="147">
@@ -5961,7 +5980,7 @@
         <v>6.2</v>
       </c>
       <c r="D147" t="n">
-        <v>0.2328904567233724</v>
+        <v>0.2328904567233725</v>
       </c>
     </row>
     <row r="148">
@@ -6057,7 +6076,7 @@
         <v>5.9</v>
       </c>
       <c r="D153" t="n">
-        <v>0.2265726951791927</v>
+        <v>0.2265726951791928</v>
       </c>
     </row>
     <row r="154">
@@ -6089,7 +6108,7 @@
         <v>5.6</v>
       </c>
       <c r="D155" t="n">
-        <v>0.2207881384697673</v>
+        <v>0.2207881384697674</v>
       </c>
     </row>
     <row r="156">
@@ -6105,7 +6124,7 @@
         <v>5.5</v>
       </c>
       <c r="D156" t="n">
-        <v>0.2253823067762057</v>
+        <v>0.2253823067762058</v>
       </c>
     </row>
     <row r="157">
@@ -6121,7 +6140,7 @@
         <v>5.5</v>
       </c>
       <c r="D157" t="n">
-        <v>0.2291800617182596</v>
+        <v>0.2291800617182597</v>
       </c>
     </row>
     <row r="158">
@@ -6137,7 +6156,7 @@
         <v>5.4</v>
       </c>
       <c r="D158" t="n">
-        <v>0.2309754226259296</v>
+        <v>0.2309754226259297</v>
       </c>
     </row>
     <row r="159">
@@ -6153,7 +6172,7 @@
         <v>5.5</v>
       </c>
       <c r="D159" t="n">
-        <v>0.2314148940180175</v>
+        <v>0.2314148940180176</v>
       </c>
     </row>
     <row r="160">
@@ -6361,7 +6380,7 @@
         <v>6.2</v>
       </c>
       <c r="D172" t="n">
-        <v>0.242646802989417</v>
+        <v>0.2426468029894171</v>
       </c>
     </row>
     <row r="173">
@@ -6393,7 +6412,7 @@
         <v>6.5</v>
       </c>
       <c r="D174" t="n">
-        <v>0.2433142716617251</v>
+        <v>0.2433142716617252</v>
       </c>
     </row>
     <row r="175">
@@ -6409,7 +6428,7 @@
         <v>6.8</v>
       </c>
       <c r="D175" t="n">
-        <v>0.2445324170963496</v>
+        <v>0.2445324170963497</v>
       </c>
     </row>
     <row r="176">
@@ -6425,7 +6444,7 @@
         <v>6.7</v>
       </c>
       <c r="D176" t="n">
-        <v>0.2458421710504726</v>
+        <v>0.2458421710504727</v>
       </c>
     </row>
     <row r="177">
@@ -6489,7 +6508,7 @@
         <v>6.9</v>
       </c>
       <c r="D180" t="n">
-        <v>0.2473780901728729</v>
+        <v>0.2474092835719974</v>
       </c>
     </row>
     <row r="181">
@@ -6499,13 +6518,29 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>29.7</v>
+        <v>29.6</v>
       </c>
       <c r="C181" t="n">
         <v>7.2</v>
       </c>
       <c r="D181" t="n">
-        <v>0.2513878650925042</v>
+        <v>0.2514723625654082</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="C182" t="n">
+        <v>7</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0.2483289996014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: update IDC to 202607 BCB release (May-2026)
IDC recedes to 0.981 (vs 0.990 in Apr-2026) as lower Q offsets higher C and I.
</commit_message>
<xml_diff>
--- a/data/processed/idc_data.xlsx
+++ b/data/processed/idc_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3605,10 +3605,10 @@
         <v>0.9393939393939393</v>
       </c>
       <c r="D182" t="n">
-        <v>0.9534926259476181</v>
+        <v>0.9532678679451505</v>
       </c>
       <c r="E182" t="n">
-        <v>0.9603739531530681</v>
+        <v>0.9602990338189121</v>
       </c>
     </row>
     <row r="183">
@@ -3618,16 +3618,35 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.9882352941176469</v>
+        <v>1</v>
       </c>
       <c r="C183" t="n">
         <v>1</v>
       </c>
       <c r="D183" t="n">
-        <v>0.9712501816740463</v>
+        <v>0.9710636030967117</v>
       </c>
       <c r="E183" t="n">
-        <v>0.986495158597231</v>
+        <v>0.9903545343655705</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>1</v>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="n">
+        <v>0.9436946533708811</v>
+      </c>
+      <c r="E184" t="n">
+        <v>0.981231551123627</v>
       </c>
     </row>
   </sheetData>
@@ -3641,7 +3660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:D184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6521,7 +6540,7 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>28.3</v>
+        <v>28.2</v>
       </c>
       <c r="C180" t="n">
         <v>7.2</v>
@@ -6543,7 +6562,7 @@
         <v>7.4</v>
       </c>
       <c r="D181" t="n">
-        <v>0.2514689798394417</v>
+        <v>0.2514593636361441</v>
       </c>
     </row>
     <row r="182">
@@ -6559,7 +6578,7 @@
         <v>7.2</v>
       </c>
       <c r="D182" t="n">
-        <v>0.2482915491357856</v>
+        <v>0.2482670266247457</v>
       </c>
     </row>
     <row r="183">
@@ -6569,13 +6588,29 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="C183" t="n">
         <v>7.4</v>
       </c>
       <c r="D183" t="n">
-        <v>0.2495047632536906</v>
+        <v>0.2494826780720774</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="C184" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D184" t="n">
+        <v>0.2476130670072468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>